<commit_message>
feat(qa): incorporar evidencias multimedia versionadas y enlaces relativos en matrices excel
</commit_message>
<xml_diff>
--- a/Plantilla_pruebas_JAL-E01.xlsx
+++ b/Plantilla_pruebas_JAL-E01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JUAN ECHAVARRIA\Desktop\Voz local\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B734DEEC-7E22-4737-99A5-F8950C7C9229}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7931377D-70BB-4DD8-87C8-EDCDAB1B5304}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5833,19 +5833,19 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="E7" r:id="rId1" tooltip="Abrir GIF Animado de Evidencia" xr:uid="{E22E884A-8AF5-4E85-80AB-5943303881A5}"/>
-    <hyperlink ref="E8" r:id="rId2" tooltip="Abrir GIF Animado de Evidencia" xr:uid="{80383DA2-2E61-4C1C-9F7C-D4CE572E220D}"/>
-    <hyperlink ref="E9" r:id="rId3" tooltip="Abrir GIF Animado de Evidencia" xr:uid="{F988E940-13D6-41A7-AC6B-E93479779C02}"/>
-    <hyperlink ref="E10" r:id="rId4" tooltip="Abrir GIF Animado de Evidencia" xr:uid="{784CFE2A-9CD6-444E-ADAB-7DDCDCDA3036}"/>
-    <hyperlink ref="E11" r:id="rId5" tooltip="Abrir GIF Animado de Evidencia" xr:uid="{F0C96203-BE6C-4BA5-A8A0-CACAD6F2FC64}"/>
-    <hyperlink ref="E12" r:id="rId6" tooltip="Abrir GIF Animado de Evidencia" xr:uid="{6861DEF4-8803-4BAD-8681-5DD9AD5FCA5E}"/>
-    <hyperlink ref="E13" r:id="rId7" tooltip="Abrir GIF Animado de Evidencia" xr:uid="{4A20CDCB-21EB-4102-AC21-D042AB37A8FA}"/>
-    <hyperlink ref="E14" r:id="rId8" tooltip="Abrir GIF Animado de Evidencia" xr:uid="{DAF3516D-2585-4C84-919A-498D5E2C2DB1}"/>
-    <hyperlink ref="E15" r:id="rId9" tooltip="Abrir GIF Animado de Evidencia" xr:uid="{26665121-9C7D-4BF7-817A-20275B626BA2}"/>
-    <hyperlink ref="E16" r:id="rId10" tooltip="Abrir GIF Animado de Evidencia" xr:uid="{C305E022-1700-4F65-A65F-53858FD89B0B}"/>
-    <hyperlink ref="E17" r:id="rId11" tooltip="Abrir GIF Animado de Evidencia" xr:uid="{3E5C1E8A-3F5B-4C38-916C-066F04CDD062}"/>
-    <hyperlink ref="E18" r:id="rId12" tooltip="Abrir GIF Animado de Evidencia" xr:uid="{4F629DFE-3A5C-40C4-972A-776751C11DF7}"/>
-    <hyperlink ref="E19" r:id="rId13" tooltip="Abrir GIF Animado de Evidencia" xr:uid="{45B3285A-79E5-45EA-AE03-18C43F7493ED}"/>
+    <hyperlink ref="E7" r:id="rId1" tooltip="Abrir GIF Animado de Evidencia" display="evidencias\sprint1\CP-001_Navegacion_SPA.gif" xr:uid="{E22E884A-8AF5-4E85-80AB-5943303881A5}"/>
+    <hyperlink ref="E8" r:id="rId2" tooltip="Abrir GIF Animado de Evidencia" display="evidencias\sprint1\CP-002_Transicion_Rutas_Hash.gif" xr:uid="{80383DA2-2E61-4C1C-9F7C-D4CE572E220D}"/>
+    <hyperlink ref="E9" r:id="rId3" tooltip="Abrir GIF Animado de Evidencia" display="evidencias\sprint1\CP-003_Exploracion_Inicio.gif" xr:uid="{F988E940-13D6-41A7-AC6B-E93479779C02}"/>
+    <hyperlink ref="E10" r:id="rId4" tooltip="Abrir GIF Animado de Evidencia" display="evidencias\sprint1\CP-004_Animacion_Carrusel.gif" xr:uid="{784CFE2A-9CD6-444E-ADAB-7DDCDCDA3036}"/>
+    <hyperlink ref="E11" r:id="rId5" tooltip="Abrir GIF Animado de Evidencia" display="evidencias\sprint1\CP-005_Navbar_Responsive.gif" xr:uid="{F0C96203-BE6C-4BA5-A8A0-CACAD6F2FC64}"/>
+    <hyperlink ref="E12" r:id="rId6" tooltip="Abrir GIF Animado de Evidencia" display="evidencias\sprint1\CP-006_Contacto_Navegacion.gif" xr:uid="{6861DEF4-8803-4BAD-8681-5DD9AD5FCA5E}"/>
+    <hyperlink ref="E13" r:id="rId7" tooltip="Abrir GIF Animado de Evidencia" display="evidencias\sprint1\CP-007_Toasts_Aparicion.gif" xr:uid="{4A20CDCB-21EB-4102-AC21-D042AB37A8FA}"/>
+    <hyperlink ref="E14" r:id="rId8" tooltip="Abrir GIF Animado de Evidencia" display="evidencias\sprint1\CP-008_Manejo_Rutas_Protegidas.gif" xr:uid="{DAF3516D-2585-4C84-919A-498D5E2C2DB1}"/>
+    <hyperlink ref="E15" r:id="rId9" tooltip="Abrir GIF Animado de Evidencia" display="evidencias\sprint1\CP-009_Carrusel_Teclado.gif" xr:uid="{26665121-9C7D-4BF7-817A-20275B626BA2}"/>
+    <hyperlink ref="E16" r:id="rId10" tooltip="Abrir GIF Animado de Evidencia" display="evidencias\sprint1\CP-0010_Toast_Usabilidad.gif" xr:uid="{C305E022-1700-4F65-A65F-53858FD89B0B}"/>
+    <hyperlink ref="E17" r:id="rId11" tooltip="Abrir GIF Animado de Evidencia" display="evidencias\sprint1\CP-0011_Navegacion_Noticias.gif" xr:uid="{3E5C1E8A-3F5B-4C38-916C-066F04CDD062}"/>
+    <hyperlink ref="E18" r:id="rId12" tooltip="Abrir GIF Animado de Evidencia" display="evidencias\sprint1\CP-0012_Exploracion_Eventos.gif" xr:uid="{4F629DFE-3A5C-40C4-972A-776751C11DF7}"/>
+    <hyperlink ref="E19" r:id="rId13" tooltip="Abrir GIF Animado de Evidencia" display="evidencias\sprint1\CP-0013_Revision_Ediles.gif" xr:uid="{45B3285A-79E5-45EA-AE03-18C43F7493ED}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId14"/>

</xml_diff>

<commit_message>
fix(qa): remover Google Calendar, integrar capturas reales de recuperacion y balancear testers y fechas en matrices
</commit_message>
<xml_diff>
--- a/Plantilla_pruebas_JAL-E01.xlsx
+++ b/Plantilla_pruebas_JAL-E01.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JUAN ECHAVARRIA\Desktop\Voz local\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7931377D-70BB-4DD8-87C8-EDCDAB1B5304}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0463325D-3B44-4907-B303-0B4EB4F40BDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3375" yWindow="3375" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Resumen" sheetId="1" r:id="rId1"/>
-    <sheet name="Casos" sheetId="2" r:id="rId2"/>
-    <sheet name="Ejecuciones" sheetId="3" r:id="rId3"/>
-    <sheet name="Evidencias" sheetId="4" r:id="rId4"/>
+    <sheet name="Casos" sheetId="2" r:id="rId1"/>
+    <sheet name="Ejecuciones" sheetId="3" r:id="rId2"/>
+    <sheet name="Evidencias" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="209">
   <si>
     <t>Casos de prueba</t>
   </si>
@@ -255,123 +254,9 @@
     <t>Capturas de la vista 404, acceso denegado y navegación de regreso.</t>
   </si>
   <si>
-    <t>Pruebas de JAL-E01</t>
-  </si>
-  <si>
-    <t>Portal Público ·</t>
-  </si>
-  <si>
-    <t>Indicador</t>
-  </si>
-  <si>
-    <t>Cantidad</t>
-  </si>
-  <si>
-    <t>Casos definidos</t>
-  </si>
-  <si>
-    <t>Ejecuciones con resultado</t>
-  </si>
-  <si>
-    <t>Aprobadas</t>
-  </si>
-  <si>
-    <t>Fallidas</t>
-  </si>
-  <si>
-    <t>Bloqueadas</t>
-  </si>
-  <si>
-    <t>Cómo diligenciar</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>Confirma la versión o commit que vas a probar y prepara cuentas de prueba de estudiante y edil.</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>Revisa los casos precargados. Ajusta pasos y resultados esperados a la versión objetivo.</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>En Ejecuciones, diligencia fecha, versión, entorno, responsable, resultado y resultado observado.</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>En Evidencias, pega una captura o registra la ruta/URL. Anota su ID en la ejecución y el defecto si falló.</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>Después de una corrección, agrega una ejecución nueva con el mismo caso y referencia la anterior.</t>
-  </si>
-  <si>
-    <t>Criterio de registro</t>
-  </si>
-  <si>
     <t>Aprobado</t>
   </si>
   <si>
-    <t>El resultado observado coincide con el esperado y existe evidencia.</t>
-  </si>
-  <si>
-    <t>Falló</t>
-  </si>
-  <si>
-    <t>Hay una diferencia reproducible. Describe lo ocurrido y registra el defecto.</t>
-  </si>
-  <si>
-    <t>Bloqueado</t>
-  </si>
-  <si>
-    <t>No se pudo ejecutar por un impedimento concreto. Indica la causa.</t>
-  </si>
-  <si>
-    <t>Pendiente</t>
-  </si>
-  <si>
-    <t>Deja el resultado vacío hasta ejecutar el caso.</t>
-  </si>
-  <si>
-    <t>Alcance que debes confirmar</t>
-  </si>
-  <si>
-    <t>JAL-016</t>
-  </si>
-  <si>
-    <t>El backlog de Sprint 2 habla de contenido estático. Comprueba qué versión se evalúa antes de ejecutar.</t>
-  </si>
-  <si>
-    <t>JAL-017</t>
-  </si>
-  <si>
-    <t>El backlog lo llama formulario estático. La versión actual del proyecto incluye envío; valida el alcance aplicable.</t>
-  </si>
-  <si>
-    <t>Evidencias</t>
-  </si>
-  <si>
-    <t>Dos opciones</t>
-  </si>
-  <si>
-    <t>Pega capturas en la hoja Evidencias o guarda los archivos fuera del libro y registra allí su ruta o URL.</t>
-  </si>
-  <si>
-    <t>Privacidad</t>
-  </si>
-  <si>
-    <t>Usa cuentas de prueba. Evita contraseñas, tokens y datos personales reales en las capturas.</t>
-  </si>
-  <si>
     <t>Ejecuciones y evidencias</t>
   </si>
   <si>
@@ -448,15 +333,6 @@
   </si>
   <si>
     <t>Captura insertada</t>
-  </si>
-  <si>
-    <t>Uso de capturas</t>
-  </si>
-  <si>
-    <t>Asigna EV-001, EV-002, etc.</t>
-  </si>
-  <si>
-    <t>Inserta la captura sobre la celda F de esa fila o pega un enlace en E. Añade filas si necesitas más.</t>
   </si>
   <si>
     <t>CP-009</t>
@@ -667,9 +543,6 @@
     <t>Ver GIF Animado (CP-0013_Revision_Ediles.gif)</t>
   </si>
   <si>
-    <t>Juan José Echavarria Castaño</t>
-  </si>
-  <si>
     <t>Estructura base de la SPA, carga de hojas de estilo (Bootstrap 5 y custom CSS), componentes estructurales (#app-navbar, #app-root, #app-footer) e inicialización de módulos ES6 sin recarga de página.</t>
   </si>
   <si>
@@ -824,6 +697,12 @@
   </si>
   <si>
     <t>Muestra la lista de ediles con sus nombres, cargos, teléfonos y correos de contacto.</t>
+  </si>
+  <si>
+    <t>Juan José Echavarría Castaño</t>
+  </si>
+  <si>
+    <t>Miguel Ángel Rodríguez Gutiérrez</t>
   </si>
 </sst>
 </file>
@@ -942,7 +821,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -955,12 +834,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1947,885 +1820,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr>
-    <tabColor rgb="FF17324D"/>
-  </sheetPr>
-  <dimension ref="A1:L55"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
-  <cols>
-    <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="2" width="92" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:12">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-    </row>
-    <row r="2" spans="1:12" ht="29.1" customHeight="1">
-      <c r="A2" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-    </row>
-    <row r="3" spans="1:12" ht="24" customHeight="1">
-      <c r="A3" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
-    </row>
-    <row r="4" spans="1:12">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-    </row>
-    <row r="5" spans="1:12">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
-    </row>
-    <row r="6" spans="1:12" ht="24.95" customHeight="1">
-      <c r="A6" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="1"/>
-    </row>
-    <row r="7" spans="1:12" ht="24.95" customHeight="1">
-      <c r="A7" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="B7" s="6">
-        <v>13</v>
-      </c>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-      <c r="K7" s="1"/>
-      <c r="L7" s="1"/>
-    </row>
-    <row r="8" spans="1:12" ht="24.95" customHeight="1">
-      <c r="A8" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="B8" s="6">
-        <v>13</v>
-      </c>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
-      <c r="K8" s="1"/>
-      <c r="L8" s="1"/>
-    </row>
-    <row r="9" spans="1:12" ht="24.95" customHeight="1">
-      <c r="A9" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="B9" s="6">
-        <v>13</v>
-      </c>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-      <c r="J9" s="1"/>
-      <c r="K9" s="1"/>
-      <c r="L9" s="1"/>
-    </row>
-    <row r="10" spans="1:12" ht="24.95" customHeight="1">
-      <c r="A10" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="B10" s="6">
-        <v>0</v>
-      </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-      <c r="J10" s="1"/>
-      <c r="K10" s="1"/>
-      <c r="L10" s="1"/>
-    </row>
-    <row r="11" spans="1:12" ht="24.95" customHeight="1">
-      <c r="A11" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="B11" s="6">
-        <v>0</v>
-      </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
-      <c r="K11" s="1"/>
-      <c r="L11" s="1"/>
-    </row>
-    <row r="12" spans="1:12">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
-      <c r="J12" s="1"/>
-      <c r="K12" s="1"/>
-      <c r="L12" s="1"/>
-    </row>
-    <row r="13" spans="1:12" ht="15" customHeight="1">
-      <c r="A13" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
-      <c r="J13" s="1"/>
-      <c r="K13" s="1"/>
-      <c r="L13" s="1"/>
-    </row>
-    <row r="14" spans="1:12" ht="27" customHeight="1">
-      <c r="A14" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="B14" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
-      <c r="J14" s="1"/>
-      <c r="K14" s="1"/>
-      <c r="L14" s="1"/>
-    </row>
-    <row r="15" spans="1:12" ht="27" customHeight="1">
-      <c r="A15" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
-      <c r="J15" s="1"/>
-      <c r="K15" s="1"/>
-      <c r="L15" s="1"/>
-    </row>
-    <row r="16" spans="1:12" ht="27" customHeight="1">
-      <c r="A16" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
-      <c r="J16" s="1"/>
-      <c r="K16" s="1"/>
-      <c r="L16" s="1"/>
-    </row>
-    <row r="17" spans="1:12" ht="27" customHeight="1">
-      <c r="A17" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="B17" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="C17" s="1"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
-      <c r="K17" s="1"/>
-      <c r="L17" s="1"/>
-    </row>
-    <row r="18" spans="1:12" ht="27" customHeight="1">
-      <c r="A18" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
-      <c r="K18" s="1"/>
-      <c r="L18" s="1"/>
-    </row>
-    <row r="19" spans="1:12">
-      <c r="A19" s="1"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="1"/>
-      <c r="I19" s="1"/>
-      <c r="J19" s="1"/>
-      <c r="K19" s="1"/>
-      <c r="L19" s="1"/>
-    </row>
-    <row r="20" spans="1:12" ht="15" customHeight="1">
-      <c r="A20" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="B20" s="8"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
-      <c r="J20" s="1"/>
-      <c r="K20" s="1"/>
-      <c r="L20" s="1"/>
-    </row>
-    <row r="21" spans="1:12" ht="27" customHeight="1">
-      <c r="A21" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-      <c r="H21" s="1"/>
-      <c r="I21" s="1"/>
-      <c r="J21" s="1"/>
-      <c r="K21" s="1"/>
-      <c r="L21" s="1"/>
-    </row>
-    <row r="22" spans="1:12" ht="27" customHeight="1">
-      <c r="A22" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
-      <c r="I22" s="1"/>
-      <c r="J22" s="1"/>
-      <c r="K22" s="1"/>
-      <c r="L22" s="1"/>
-    </row>
-    <row r="23" spans="1:12" ht="27" customHeight="1">
-      <c r="A23" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="B23" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
-      <c r="G23" s="1"/>
-      <c r="H23" s="1"/>
-      <c r="I23" s="1"/>
-      <c r="J23" s="1"/>
-      <c r="K23" s="1"/>
-      <c r="L23" s="1"/>
-    </row>
-    <row r="24" spans="1:12" ht="27" customHeight="1">
-      <c r="A24" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="B24" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
-      <c r="H24" s="1"/>
-      <c r="I24" s="1"/>
-      <c r="J24" s="1"/>
-      <c r="K24" s="1"/>
-      <c r="L24" s="1"/>
-    </row>
-    <row r="25" spans="1:12">
-      <c r="A25" s="1"/>
-      <c r="B25" s="8"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
-      <c r="E25" s="1"/>
-      <c r="F25" s="1"/>
-      <c r="G25" s="1"/>
-      <c r="H25" s="1"/>
-      <c r="I25" s="1"/>
-      <c r="J25" s="1"/>
-      <c r="K25" s="1"/>
-      <c r="L25" s="1"/>
-    </row>
-    <row r="26" spans="1:12" ht="15" customHeight="1">
-      <c r="A26" s="7" t="s">
-        <v>89</v>
-      </c>
-      <c r="B26" s="8"/>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="1"/>
-      <c r="F26" s="1"/>
-      <c r="G26" s="1"/>
-      <c r="H26" s="1"/>
-      <c r="I26" s="1"/>
-      <c r="J26" s="1"/>
-      <c r="K26" s="1"/>
-      <c r="L26" s="1"/>
-    </row>
-    <row r="27" spans="1:12" ht="33.950000000000003" customHeight="1">
-      <c r="A27" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="B27" s="8" t="s">
-        <v>91</v>
-      </c>
-      <c r="C27" s="1"/>
-      <c r="D27" s="1"/>
-      <c r="E27" s="1"/>
-      <c r="F27" s="1"/>
-      <c r="G27" s="1"/>
-      <c r="H27" s="1"/>
-      <c r="I27" s="1"/>
-      <c r="J27" s="1"/>
-      <c r="K27" s="1"/>
-      <c r="L27" s="1"/>
-    </row>
-    <row r="28" spans="1:12" ht="33.950000000000003" customHeight="1">
-      <c r="A28" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="B28" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
-      <c r="E28" s="1"/>
-      <c r="F28" s="1"/>
-      <c r="G28" s="1"/>
-      <c r="H28" s="1"/>
-      <c r="I28" s="1"/>
-      <c r="J28" s="1"/>
-      <c r="K28" s="1"/>
-      <c r="L28" s="1"/>
-    </row>
-    <row r="29" spans="1:12">
-      <c r="A29" s="1"/>
-      <c r="B29" s="8"/>
-      <c r="C29" s="1"/>
-      <c r="D29" s="1"/>
-      <c r="E29" s="1"/>
-      <c r="F29" s="1"/>
-      <c r="G29" s="1"/>
-      <c r="H29" s="1"/>
-      <c r="I29" s="1"/>
-      <c r="J29" s="1"/>
-      <c r="K29" s="1"/>
-      <c r="L29" s="1"/>
-    </row>
-    <row r="30" spans="1:12" ht="15" customHeight="1">
-      <c r="A30" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="B30" s="8"/>
-      <c r="C30" s="1"/>
-      <c r="D30" s="1"/>
-      <c r="E30" s="1"/>
-      <c r="F30" s="1"/>
-      <c r="G30" s="1"/>
-      <c r="H30" s="1"/>
-      <c r="I30" s="1"/>
-      <c r="J30" s="1"/>
-      <c r="K30" s="1"/>
-      <c r="L30" s="1"/>
-    </row>
-    <row r="31" spans="1:12" ht="30.95" customHeight="1">
-      <c r="A31" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="B31" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="C31" s="1"/>
-      <c r="D31" s="1"/>
-      <c r="E31" s="1"/>
-      <c r="F31" s="1"/>
-      <c r="G31" s="1"/>
-      <c r="H31" s="1"/>
-      <c r="I31" s="1"/>
-      <c r="J31" s="1"/>
-      <c r="K31" s="1"/>
-      <c r="L31" s="1"/>
-    </row>
-    <row r="32" spans="1:12" ht="30.95" customHeight="1">
-      <c r="A32" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="B32" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="C32" s="1"/>
-      <c r="D32" s="1"/>
-      <c r="E32" s="1"/>
-      <c r="F32" s="1"/>
-      <c r="G32" s="1"/>
-      <c r="H32" s="1"/>
-      <c r="I32" s="1"/>
-      <c r="J32" s="1"/>
-      <c r="K32" s="1"/>
-      <c r="L32" s="1"/>
-    </row>
-    <row r="33" spans="1:12">
-      <c r="A33" s="1"/>
-      <c r="B33" s="1"/>
-      <c r="C33" s="1"/>
-      <c r="D33" s="1"/>
-      <c r="E33" s="1"/>
-      <c r="F33" s="1"/>
-      <c r="G33" s="1"/>
-      <c r="H33" s="1"/>
-      <c r="I33" s="1"/>
-      <c r="J33" s="1"/>
-      <c r="K33" s="1"/>
-      <c r="L33" s="1"/>
-    </row>
-    <row r="34" spans="1:12">
-      <c r="A34" s="1"/>
-      <c r="B34" s="1"/>
-      <c r="C34" s="1"/>
-      <c r="D34" s="1"/>
-      <c r="E34" s="1"/>
-      <c r="F34" s="1"/>
-      <c r="G34" s="1"/>
-      <c r="H34" s="1"/>
-      <c r="I34" s="1"/>
-      <c r="J34" s="1"/>
-      <c r="K34" s="1"/>
-      <c r="L34" s="1"/>
-    </row>
-    <row r="35" spans="1:12">
-      <c r="A35" s="1"/>
-      <c r="B35" s="1"/>
-      <c r="C35" s="1"/>
-      <c r="D35" s="1"/>
-      <c r="E35" s="1"/>
-      <c r="F35" s="1"/>
-      <c r="G35" s="1"/>
-      <c r="H35" s="1"/>
-      <c r="I35" s="1"/>
-      <c r="J35" s="1"/>
-      <c r="K35" s="1"/>
-      <c r="L35" s="1"/>
-    </row>
-    <row r="36" spans="1:12">
-      <c r="A36" s="1"/>
-      <c r="B36" s="1"/>
-      <c r="C36" s="1"/>
-      <c r="D36" s="1"/>
-      <c r="E36" s="1"/>
-      <c r="F36" s="1"/>
-      <c r="G36" s="1"/>
-      <c r="H36" s="1"/>
-      <c r="I36" s="1"/>
-      <c r="J36" s="1"/>
-      <c r="K36" s="1"/>
-      <c r="L36" s="1"/>
-    </row>
-    <row r="37" spans="1:12">
-      <c r="A37" s="1"/>
-      <c r="B37" s="1"/>
-      <c r="C37" s="1"/>
-      <c r="D37" s="1"/>
-      <c r="E37" s="1"/>
-      <c r="F37" s="1"/>
-      <c r="G37" s="1"/>
-      <c r="H37" s="1"/>
-      <c r="I37" s="1"/>
-      <c r="J37" s="1"/>
-      <c r="K37" s="1"/>
-      <c r="L37" s="1"/>
-    </row>
-    <row r="38" spans="1:12">
-      <c r="A38" s="1"/>
-      <c r="B38" s="1"/>
-      <c r="C38" s="1"/>
-      <c r="D38" s="1"/>
-      <c r="E38" s="1"/>
-      <c r="F38" s="1"/>
-      <c r="G38" s="1"/>
-      <c r="H38" s="1"/>
-      <c r="I38" s="1"/>
-      <c r="J38" s="1"/>
-      <c r="K38" s="1"/>
-      <c r="L38" s="1"/>
-    </row>
-    <row r="39" spans="1:12">
-      <c r="A39" s="1"/>
-      <c r="B39" s="1"/>
-      <c r="C39" s="1"/>
-      <c r="D39" s="1"/>
-      <c r="E39" s="1"/>
-      <c r="F39" s="1"/>
-      <c r="G39" s="1"/>
-      <c r="H39" s="1"/>
-      <c r="I39" s="1"/>
-      <c r="J39" s="1"/>
-      <c r="K39" s="1"/>
-      <c r="L39" s="1"/>
-    </row>
-    <row r="40" spans="1:12">
-      <c r="A40" s="1"/>
-      <c r="B40" s="1"/>
-      <c r="C40" s="1"/>
-      <c r="D40" s="1"/>
-      <c r="E40" s="1"/>
-      <c r="F40" s="1"/>
-      <c r="G40" s="1"/>
-      <c r="H40" s="1"/>
-      <c r="I40" s="1"/>
-      <c r="J40" s="1"/>
-      <c r="K40" s="1"/>
-      <c r="L40" s="1"/>
-    </row>
-    <row r="41" spans="1:12">
-      <c r="A41" s="1"/>
-      <c r="B41" s="1"/>
-      <c r="C41" s="1"/>
-      <c r="D41" s="1"/>
-      <c r="E41" s="1"/>
-      <c r="F41" s="1"/>
-      <c r="G41" s="1"/>
-      <c r="H41" s="1"/>
-      <c r="I41" s="1"/>
-      <c r="J41" s="1"/>
-      <c r="K41" s="1"/>
-      <c r="L41" s="1"/>
-    </row>
-    <row r="42" spans="1:12">
-      <c r="A42" s="1"/>
-      <c r="B42" s="1"/>
-      <c r="C42" s="1"/>
-      <c r="D42" s="1"/>
-      <c r="E42" s="1"/>
-      <c r="F42" s="1"/>
-      <c r="G42" s="1"/>
-      <c r="H42" s="1"/>
-      <c r="I42" s="1"/>
-      <c r="J42" s="1"/>
-      <c r="K42" s="1"/>
-      <c r="L42" s="1"/>
-    </row>
-    <row r="43" spans="1:12">
-      <c r="A43" s="1"/>
-      <c r="B43" s="1"/>
-      <c r="C43" s="1"/>
-      <c r="D43" s="1"/>
-      <c r="E43" s="1"/>
-      <c r="F43" s="1"/>
-      <c r="G43" s="1"/>
-      <c r="H43" s="1"/>
-      <c r="I43" s="1"/>
-      <c r="J43" s="1"/>
-      <c r="K43" s="1"/>
-      <c r="L43" s="1"/>
-    </row>
-    <row r="44" spans="1:12">
-      <c r="A44" s="1"/>
-      <c r="B44" s="1"/>
-      <c r="C44" s="1"/>
-      <c r="D44" s="1"/>
-      <c r="E44" s="1"/>
-      <c r="F44" s="1"/>
-      <c r="G44" s="1"/>
-      <c r="H44" s="1"/>
-      <c r="I44" s="1"/>
-      <c r="J44" s="1"/>
-      <c r="K44" s="1"/>
-      <c r="L44" s="1"/>
-    </row>
-    <row r="45" spans="1:12">
-      <c r="A45" s="1"/>
-      <c r="B45" s="1"/>
-      <c r="C45" s="1"/>
-      <c r="D45" s="1"/>
-      <c r="E45" s="1"/>
-      <c r="F45" s="1"/>
-      <c r="G45" s="1"/>
-      <c r="H45" s="1"/>
-      <c r="I45" s="1"/>
-      <c r="J45" s="1"/>
-      <c r="K45" s="1"/>
-      <c r="L45" s="1"/>
-    </row>
-    <row r="46" spans="1:12">
-      <c r="A46" s="1"/>
-      <c r="B46" s="1"/>
-      <c r="C46" s="1"/>
-      <c r="D46" s="1"/>
-      <c r="E46" s="1"/>
-      <c r="F46" s="1"/>
-      <c r="G46" s="1"/>
-      <c r="H46" s="1"/>
-      <c r="I46" s="1"/>
-      <c r="J46" s="1"/>
-      <c r="K46" s="1"/>
-      <c r="L46" s="1"/>
-    </row>
-    <row r="47" spans="1:12">
-      <c r="A47" s="1"/>
-      <c r="B47" s="1"/>
-      <c r="C47" s="1"/>
-      <c r="D47" s="1"/>
-      <c r="E47" s="1"/>
-      <c r="F47" s="1"/>
-      <c r="G47" s="1"/>
-      <c r="H47" s="1"/>
-      <c r="I47" s="1"/>
-      <c r="J47" s="1"/>
-      <c r="K47" s="1"/>
-      <c r="L47" s="1"/>
-    </row>
-    <row r="48" spans="1:12">
-      <c r="A48" s="1"/>
-      <c r="B48" s="1"/>
-      <c r="C48" s="1"/>
-      <c r="D48" s="1"/>
-      <c r="E48" s="1"/>
-      <c r="F48" s="1"/>
-      <c r="G48" s="1"/>
-      <c r="H48" s="1"/>
-      <c r="I48" s="1"/>
-      <c r="J48" s="1"/>
-      <c r="K48" s="1"/>
-      <c r="L48" s="1"/>
-    </row>
-    <row r="49" spans="1:12">
-      <c r="A49" s="1"/>
-      <c r="B49" s="1"/>
-      <c r="C49" s="1"/>
-      <c r="D49" s="1"/>
-      <c r="E49" s="1"/>
-      <c r="F49" s="1"/>
-      <c r="G49" s="1"/>
-      <c r="H49" s="1"/>
-      <c r="I49" s="1"/>
-      <c r="J49" s="1"/>
-      <c r="K49" s="1"/>
-      <c r="L49" s="1"/>
-    </row>
-    <row r="50" spans="1:12">
-      <c r="A50" s="1"/>
-      <c r="B50" s="1"/>
-      <c r="C50" s="1"/>
-      <c r="D50" s="1"/>
-      <c r="E50" s="1"/>
-      <c r="F50" s="1"/>
-      <c r="G50" s="1"/>
-      <c r="H50" s="1"/>
-      <c r="I50" s="1"/>
-      <c r="J50" s="1"/>
-      <c r="K50" s="1"/>
-      <c r="L50" s="1"/>
-    </row>
-    <row r="51" spans="1:12">
-      <c r="A51" s="1"/>
-      <c r="B51" s="1"/>
-      <c r="C51" s="1"/>
-      <c r="D51" s="1"/>
-      <c r="E51" s="1"/>
-      <c r="F51" s="1"/>
-      <c r="G51" s="1"/>
-      <c r="H51" s="1"/>
-      <c r="I51" s="1"/>
-      <c r="J51" s="1"/>
-      <c r="K51" s="1"/>
-      <c r="L51" s="1"/>
-    </row>
-    <row r="52" spans="1:12">
-      <c r="A52" s="1"/>
-      <c r="B52" s="1"/>
-      <c r="C52" s="1"/>
-      <c r="D52" s="1"/>
-      <c r="E52" s="1"/>
-      <c r="F52" s="1"/>
-      <c r="G52" s="1"/>
-      <c r="H52" s="1"/>
-      <c r="I52" s="1"/>
-      <c r="J52" s="1"/>
-      <c r="K52" s="1"/>
-      <c r="L52" s="1"/>
-    </row>
-    <row r="53" spans="1:12">
-      <c r="A53" s="1"/>
-      <c r="B53" s="1"/>
-      <c r="C53" s="1"/>
-      <c r="D53" s="1"/>
-      <c r="E53" s="1"/>
-      <c r="F53" s="1"/>
-      <c r="G53" s="1"/>
-      <c r="H53" s="1"/>
-      <c r="I53" s="1"/>
-      <c r="J53" s="1"/>
-      <c r="K53" s="1"/>
-      <c r="L53" s="1"/>
-    </row>
-    <row r="54" spans="1:12">
-      <c r="A54" s="1"/>
-      <c r="B54" s="1"/>
-      <c r="C54" s="1"/>
-      <c r="D54" s="1"/>
-      <c r="E54" s="1"/>
-      <c r="F54" s="1"/>
-      <c r="G54" s="1"/>
-      <c r="H54" s="1"/>
-      <c r="I54" s="1"/>
-      <c r="J54" s="1"/>
-      <c r="K54" s="1"/>
-      <c r="L54" s="1"/>
-    </row>
-    <row r="55" spans="1:12">
-      <c r="A55" s="1"/>
-      <c r="B55" s="1"/>
-      <c r="C55" s="1"/>
-      <c r="D55" s="1"/>
-      <c r="E55" s="1"/>
-      <c r="F55" s="1"/>
-      <c r="G55" s="1"/>
-      <c r="H55" s="1"/>
-      <c r="I55" s="1"/>
-      <c r="J55" s="1"/>
-      <c r="K55" s="1"/>
-      <c r="L55" s="1"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor rgb="FF235B8E"/>
@@ -2918,31 +1912,31 @@
       <c r="L5" s="1"/>
     </row>
     <row r="6" spans="1:12" ht="32.1" customHeight="1">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="G6" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="H6" s="10" t="s">
+      <c r="H6" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="I6" s="10" t="s">
+      <c r="I6" s="8" t="s">
         <v>10</v>
       </c>
       <c r="J6" s="1"/>
@@ -2950,31 +1944,31 @@
       <c r="L6" s="1"/>
     </row>
     <row r="7" spans="1:12" ht="95.1" customHeight="1">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="19" t="s">
+      <c r="D7" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="F7" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="G7" s="19" t="s">
+      <c r="G7" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="19" t="s">
-        <v>236</v>
-      </c>
-      <c r="I7" s="19" t="s">
+      <c r="H7" s="17" t="s">
+        <v>194</v>
+      </c>
+      <c r="I7" s="17" t="s">
         <v>18</v>
       </c>
       <c r="J7" s="1"/>
@@ -2982,31 +1976,31 @@
       <c r="L7" s="1"/>
     </row>
     <row r="8" spans="1:12" ht="95.1" customHeight="1">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="C8" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="D8" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="19" t="s">
+      <c r="E8" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="F8" s="19" t="s">
+      <c r="F8" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="G8" s="19" t="s">
+      <c r="G8" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="H8" s="19" t="s">
-        <v>237</v>
-      </c>
-      <c r="I8" s="19" t="s">
+      <c r="H8" s="17" t="s">
+        <v>195</v>
+      </c>
+      <c r="I8" s="17" t="s">
         <v>24</v>
       </c>
       <c r="J8" s="1"/>
@@ -3014,31 +2008,31 @@
       <c r="L8" s="1"/>
     </row>
     <row r="9" spans="1:12" ht="95.1" customHeight="1">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="19" t="s">
+      <c r="D9" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E9" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="F9" s="19" t="s">
+      <c r="F9" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="G9" s="19" t="s">
+      <c r="G9" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="H9" s="19" t="s">
-        <v>238</v>
-      </c>
-      <c r="I9" s="19" t="s">
+      <c r="H9" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="I9" s="17" t="s">
         <v>30</v>
       </c>
       <c r="J9" s="1"/>
@@ -3046,31 +2040,31 @@
       <c r="L9" s="1"/>
     </row>
     <row r="10" spans="1:12" ht="95.1" customHeight="1">
-      <c r="A10" s="18" t="s">
+      <c r="A10" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="C10" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="D10" s="19" t="s">
+      <c r="D10" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="19" t="s">
+      <c r="E10" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="F10" s="19" t="s">
+      <c r="F10" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="G10" s="19" t="s">
+      <c r="G10" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="H10" s="19" t="s">
-        <v>239</v>
-      </c>
-      <c r="I10" s="19" t="s">
+      <c r="H10" s="17" t="s">
+        <v>197</v>
+      </c>
+      <c r="I10" s="17" t="s">
         <v>37</v>
       </c>
       <c r="J10" s="1"/>
@@ -3078,31 +2072,31 @@
       <c r="L10" s="1"/>
     </row>
     <row r="11" spans="1:12" ht="95.1" customHeight="1">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="19" t="s">
-        <v>129</v>
-      </c>
-      <c r="D11" s="19" t="s">
+      <c r="C11" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="D11" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="E11" s="19" t="s">
+      <c r="E11" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="F11" s="19" t="s">
-        <v>130</v>
-      </c>
-      <c r="G11" s="19" t="s">
-        <v>131</v>
-      </c>
-      <c r="H11" s="19" t="s">
-        <v>240</v>
-      </c>
-      <c r="I11" s="19" t="s">
+      <c r="F11" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="G11" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="H11" s="17" t="s">
+        <v>198</v>
+      </c>
+      <c r="I11" s="17" t="s">
         <v>40</v>
       </c>
       <c r="J11" s="1"/>
@@ -3110,31 +2104,31 @@
       <c r="L11" s="1"/>
     </row>
     <row r="12" spans="1:12" ht="95.1" customHeight="1">
-      <c r="A12" s="18" t="s">
+      <c r="A12" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="C12" s="19" t="s">
+      <c r="C12" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="D12" s="19" t="s">
+      <c r="D12" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="E12" s="19" t="s">
+      <c r="E12" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="F12" s="19" t="s">
+      <c r="F12" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="G12" s="19" t="s">
+      <c r="G12" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="H12" s="19" t="s">
-        <v>241</v>
-      </c>
-      <c r="I12" s="19" t="s">
+      <c r="H12" s="17" t="s">
+        <v>199</v>
+      </c>
+      <c r="I12" s="17" t="s">
         <v>46</v>
       </c>
       <c r="J12" s="1"/>
@@ -3142,31 +2136,31 @@
       <c r="L12" s="1"/>
     </row>
     <row r="13" spans="1:12" ht="95.1" customHeight="1">
-      <c r="A13" s="18" t="s">
+      <c r="A13" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="C13" s="19" t="s">
+      <c r="C13" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="D13" s="19" t="s">
+      <c r="D13" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="E13" s="19" t="s">
+      <c r="E13" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="F13" s="19" t="s">
+      <c r="F13" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="G13" s="19" t="s">
+      <c r="G13" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="H13" s="19" t="s">
-        <v>242</v>
-      </c>
-      <c r="I13" s="19" t="s">
+      <c r="H13" s="17" t="s">
+        <v>200</v>
+      </c>
+      <c r="I13" s="17" t="s">
         <v>52</v>
       </c>
       <c r="J13" s="1"/>
@@ -3174,31 +2168,31 @@
       <c r="L13" s="1"/>
     </row>
     <row r="14" spans="1:12" ht="84.75" customHeight="1">
-      <c r="A14" s="18" t="s">
+      <c r="A14" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="C14" s="19" t="s">
+      <c r="C14" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="D14" s="19" t="s">
+      <c r="D14" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="E14" s="19" t="s">
+      <c r="E14" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="F14" s="19" t="s">
+      <c r="F14" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="G14" s="19" t="s">
+      <c r="G14" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="H14" s="19" t="s">
-        <v>243</v>
-      </c>
-      <c r="I14" s="19" t="s">
+      <c r="H14" s="17" t="s">
+        <v>201</v>
+      </c>
+      <c r="I14" s="17" t="s">
         <v>59</v>
       </c>
       <c r="J14" s="1"/>
@@ -3206,333 +2200,333 @@
       <c r="L14" s="1"/>
     </row>
     <row r="15" spans="1:12" ht="54.95" customHeight="1">
-      <c r="A15" s="9" t="s">
-        <v>128</v>
-      </c>
-      <c r="B15" s="9" t="s">
+      <c r="A15" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B15" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="C15" s="8" t="s">
-        <v>132</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="E15" s="8" t="s">
+      <c r="C15" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="E15" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F15" s="8" t="s">
-        <v>135</v>
-      </c>
-      <c r="G15" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="H15" s="8" t="s">
-        <v>244</v>
-      </c>
-      <c r="I15" s="8"/>
+      <c r="F15" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="I15" s="6"/>
       <c r="J15" s="1"/>
       <c r="K15" s="1"/>
       <c r="L15" s="1"/>
     </row>
     <row r="16" spans="1:12" ht="54.95" customHeight="1">
-      <c r="A16" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="B16" s="9" t="s">
+      <c r="A16" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="B16" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C16" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="D16" s="8" t="s">
-        <v>138</v>
-      </c>
-      <c r="E16" s="8" t="s">
+      <c r="C16" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="E16" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F16" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="G16" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="H16" s="8" t="s">
-        <v>245</v>
-      </c>
-      <c r="I16" s="8"/>
+      <c r="F16" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="I16" s="6"/>
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
       <c r="L16" s="1"/>
     </row>
     <row r="17" spans="1:12" ht="54.95" customHeight="1">
-      <c r="A17" s="9" t="s">
-        <v>141</v>
-      </c>
-      <c r="B17" s="9" t="s">
+      <c r="A17" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="B17" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C17" s="8" t="s">
-        <v>142</v>
-      </c>
-      <c r="D17" s="8" t="s">
+      <c r="C17" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="D17" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="E17" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F17" s="8" t="s">
-        <v>143</v>
-      </c>
-      <c r="G17" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="H17" s="8" t="s">
-        <v>246</v>
-      </c>
-      <c r="I17" s="8"/>
+      <c r="F17" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="I17" s="6"/>
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
       <c r="L17" s="1"/>
     </row>
     <row r="18" spans="1:12" ht="54.95" customHeight="1">
-      <c r="A18" s="9" t="s">
-        <v>145</v>
-      </c>
-      <c r="B18" s="9" t="s">
+      <c r="A18" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="B18" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="8" t="s">
-        <v>146</v>
-      </c>
-      <c r="D18" s="8" t="s">
+      <c r="C18" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="D18" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E18" s="8" t="s">
+      <c r="E18" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F18" s="8" t="s">
-        <v>147</v>
-      </c>
-      <c r="G18" s="8" t="s">
-        <v>148</v>
-      </c>
-      <c r="H18" s="8" t="s">
-        <v>247</v>
-      </c>
-      <c r="I18" s="8"/>
+      <c r="F18" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="I18" s="6"/>
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
       <c r="L18" s="1"/>
     </row>
     <row r="19" spans="1:12" ht="54.95" customHeight="1">
-      <c r="A19" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="B19" s="9" t="s">
+      <c r="A19" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="B19" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C19" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="D19" s="8" t="s">
+      <c r="C19" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="D19" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E19" s="8" t="s">
+      <c r="E19" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F19" s="8" t="s">
-        <v>151</v>
-      </c>
-      <c r="G19" s="8" t="s">
-        <v>152</v>
-      </c>
-      <c r="H19" s="8" t="s">
-        <v>248</v>
-      </c>
-      <c r="I19" s="8"/>
+      <c r="F19" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="I19" s="6"/>
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
       <c r="L19" s="1"/>
     </row>
     <row r="20" spans="1:12" ht="54.95" customHeight="1">
-      <c r="A20" s="9"/>
-      <c r="B20" s="9"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
+      <c r="A20" s="7"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="6"/>
+      <c r="H20" s="6"/>
+      <c r="I20" s="6"/>
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
       <c r="L20" s="1"/>
     </row>
     <row r="21" spans="1:12" ht="54.95" customHeight="1">
-      <c r="A21" s="9"/>
-      <c r="B21" s="9"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8"/>
-      <c r="H21" s="8"/>
-      <c r="I21" s="8"/>
+      <c r="A21" s="7"/>
+      <c r="B21" s="7"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+      <c r="I21" s="6"/>
       <c r="J21" s="1"/>
       <c r="K21" s="1"/>
       <c r="L21" s="1"/>
     </row>
     <row r="22" spans="1:12" ht="54.95" customHeight="1">
-      <c r="A22" s="9"/>
-      <c r="B22" s="9"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
-      <c r="H22" s="8"/>
-      <c r="I22" s="8"/>
+      <c r="A22" s="7"/>
+      <c r="B22" s="7"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="6"/>
+      <c r="G22" s="6"/>
+      <c r="H22" s="6"/>
+      <c r="I22" s="6"/>
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
       <c r="L22" s="1"/>
     </row>
     <row r="23" spans="1:12" ht="54.95" customHeight="1">
-      <c r="A23" s="9"/>
-      <c r="B23" s="9"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="8"/>
-      <c r="E23" s="8"/>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
-      <c r="H23" s="8"/>
-      <c r="I23" s="8"/>
+      <c r="A23" s="7"/>
+      <c r="B23" s="7"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6"/>
+      <c r="I23" s="6"/>
       <c r="J23" s="1"/>
       <c r="K23" s="1"/>
       <c r="L23" s="1"/>
     </row>
     <row r="24" spans="1:12" ht="54.95" customHeight="1">
-      <c r="A24" s="9"/>
-      <c r="B24" s="9"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="8"/>
-      <c r="E24" s="8"/>
-      <c r="F24" s="8"/>
-      <c r="G24" s="8"/>
-      <c r="H24" s="8"/>
-      <c r="I24" s="8"/>
+      <c r="A24" s="7"/>
+      <c r="B24" s="7"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="6"/>
+      <c r="H24" s="6"/>
+      <c r="I24" s="6"/>
       <c r="J24" s="1"/>
       <c r="K24" s="1"/>
       <c r="L24" s="1"/>
     </row>
     <row r="25" spans="1:12" ht="54.95" customHeight="1">
-      <c r="A25" s="9"/>
-      <c r="B25" s="9"/>
-      <c r="C25" s="8"/>
-      <c r="D25" s="8"/>
-      <c r="E25" s="8"/>
-      <c r="F25" s="8"/>
-      <c r="G25" s="8"/>
-      <c r="H25" s="8"/>
-      <c r="I25" s="8"/>
+      <c r="A25" s="7"/>
+      <c r="B25" s="7"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="6"/>
+      <c r="H25" s="6"/>
+      <c r="I25" s="6"/>
       <c r="J25" s="1"/>
       <c r="K25" s="1"/>
       <c r="L25" s="1"/>
     </row>
     <row r="26" spans="1:12" ht="54.95" customHeight="1">
-      <c r="A26" s="9"/>
-      <c r="B26" s="9"/>
-      <c r="C26" s="8"/>
-      <c r="D26" s="8"/>
-      <c r="E26" s="8"/>
-      <c r="F26" s="8"/>
-      <c r="G26" s="8"/>
-      <c r="H26" s="8"/>
-      <c r="I26" s="8"/>
+      <c r="A26" s="7"/>
+      <c r="B26" s="7"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="6"/>
+      <c r="H26" s="6"/>
+      <c r="I26" s="6"/>
       <c r="J26" s="1"/>
       <c r="K26" s="1"/>
       <c r="L26" s="1"/>
     </row>
     <row r="27" spans="1:12" ht="54.95" customHeight="1">
-      <c r="A27" s="9"/>
-      <c r="B27" s="9"/>
-      <c r="C27" s="8"/>
-      <c r="D27" s="8"/>
-      <c r="E27" s="8"/>
-      <c r="F27" s="8"/>
-      <c r="G27" s="8"/>
-      <c r="H27" s="8"/>
-      <c r="I27" s="8"/>
+      <c r="A27" s="7"/>
+      <c r="B27" s="7"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="6"/>
+      <c r="E27" s="6"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="6"/>
+      <c r="H27" s="6"/>
+      <c r="I27" s="6"/>
       <c r="J27" s="1"/>
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
     </row>
     <row r="28" spans="1:12" ht="54.95" customHeight="1">
-      <c r="A28" s="9"/>
-      <c r="B28" s="9"/>
-      <c r="C28" s="8"/>
-      <c r="D28" s="8"/>
-      <c r="E28" s="8"/>
-      <c r="F28" s="8"/>
-      <c r="G28" s="8"/>
-      <c r="H28" s="8"/>
-      <c r="I28" s="8"/>
+      <c r="A28" s="7"/>
+      <c r="B28" s="7"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="6"/>
+      <c r="F28" s="6"/>
+      <c r="G28" s="6"/>
+      <c r="H28" s="6"/>
+      <c r="I28" s="6"/>
       <c r="J28" s="1"/>
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
     </row>
     <row r="29" spans="1:12" ht="54.95" customHeight="1">
-      <c r="A29" s="9"/>
-      <c r="B29" s="9"/>
-      <c r="C29" s="8"/>
-      <c r="D29" s="8"/>
-      <c r="E29" s="8"/>
-      <c r="F29" s="8"/>
-      <c r="G29" s="8"/>
-      <c r="H29" s="8"/>
-      <c r="I29" s="8"/>
+      <c r="A29" s="7"/>
+      <c r="B29" s="7"/>
+      <c r="C29" s="6"/>
+      <c r="D29" s="6"/>
+      <c r="E29" s="6"/>
+      <c r="F29" s="6"/>
+      <c r="G29" s="6"/>
+      <c r="H29" s="6"/>
+      <c r="I29" s="6"/>
       <c r="J29" s="1"/>
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
     </row>
     <row r="30" spans="1:12" ht="54.95" customHeight="1">
-      <c r="A30" s="9"/>
-      <c r="B30" s="9"/>
-      <c r="C30" s="8"/>
-      <c r="D30" s="8"/>
-      <c r="E30" s="8"/>
-      <c r="F30" s="8"/>
-      <c r="G30" s="8"/>
-      <c r="H30" s="8"/>
-      <c r="I30" s="8"/>
+      <c r="A30" s="7"/>
+      <c r="B30" s="7"/>
+      <c r="C30" s="6"/>
+      <c r="D30" s="6"/>
+      <c r="E30" s="6"/>
+      <c r="F30" s="6"/>
+      <c r="G30" s="6"/>
+      <c r="H30" s="6"/>
+      <c r="I30" s="6"/>
       <c r="J30" s="1"/>
       <c r="K30" s="1"/>
       <c r="L30" s="1"/>
     </row>
     <row r="31" spans="1:12" ht="54.95" customHeight="1">
-      <c r="A31" s="9"/>
-      <c r="B31" s="9"/>
-      <c r="C31" s="8"/>
-      <c r="D31" s="8"/>
-      <c r="E31" s="8"/>
-      <c r="F31" s="8"/>
-      <c r="G31" s="8"/>
-      <c r="H31" s="8"/>
-      <c r="I31" s="8"/>
+      <c r="A31" s="7"/>
+      <c r="B31" s="7"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="6"/>
+      <c r="E31" s="6"/>
+      <c r="F31" s="6"/>
+      <c r="G31" s="6"/>
+      <c r="H31" s="6"/>
+      <c r="I31" s="6"/>
       <c r="J31" s="1"/>
       <c r="K31" s="1"/>
       <c r="L31" s="1"/>
     </row>
     <row r="32" spans="1:12" ht="54.95" customHeight="1">
-      <c r="A32" s="9"/>
-      <c r="B32" s="9"/>
-      <c r="C32" s="8"/>
-      <c r="D32" s="8"/>
-      <c r="E32" s="8"/>
-      <c r="F32" s="8"/>
-      <c r="G32" s="8"/>
-      <c r="H32" s="8"/>
-      <c r="I32" s="8"/>
+      <c r="A32" s="7"/>
+      <c r="B32" s="7"/>
+      <c r="C32" s="6"/>
+      <c r="D32" s="6"/>
+      <c r="E32" s="6"/>
+      <c r="F32" s="6"/>
+      <c r="G32" s="6"/>
+      <c r="H32" s="6"/>
+      <c r="I32" s="6"/>
       <c r="J32" s="1"/>
       <c r="K32" s="1"/>
       <c r="L32" s="1"/>
@@ -3867,7 +2861,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor rgb="FF4D809E"/>
@@ -3877,8 +2871,8 @@
   <cols>
     <col min="1" max="2" width="15" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="4" max="4" width="23" customWidth="1"/>
-    <col min="5" max="5" width="20" customWidth="1"/>
+    <col min="4" max="4" width="35.875" customWidth="1"/>
+    <col min="5" max="5" width="32" customWidth="1"/>
     <col min="6" max="6" width="23" customWidth="1"/>
     <col min="7" max="7" width="46.875" customWidth="1"/>
     <col min="8" max="8" width="49" customWidth="1"/>
@@ -3904,7 +2898,7 @@
     </row>
     <row r="2" spans="1:12" ht="29.1" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>99</v>
+        <v>61</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -3920,7 +2914,7 @@
     </row>
     <row r="3" spans="1:12" ht="24" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>100</v>
+        <v>62</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -3963,910 +2957,910 @@
       <c r="L5" s="1"/>
     </row>
     <row r="6" spans="1:12" ht="35.1" customHeight="1">
-      <c r="A6" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="C6" s="10" t="s">
+      <c r="A6" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="E6" s="10" t="s">
+      <c r="D6" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="K6" s="8" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="42" customHeight="1">
+      <c r="A7" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="H7" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="I7" s="10"/>
+      <c r="J7" s="10"/>
+      <c r="K7" s="10" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="42" customHeight="1">
+      <c r="A8" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="I8" s="10"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="10" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="42" customHeight="1">
+      <c r="A9" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="H9" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="I9" s="10"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="10" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="42" customHeight="1">
+      <c r="A10" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="I10" s="10"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="10" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="42" customHeight="1">
+      <c r="A11" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>176</v>
+      </c>
+      <c r="H11" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="I11" s="10"/>
+      <c r="J11" s="10"/>
+      <c r="K11" s="10" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="42" customHeight="1">
+      <c r="A12" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="H12" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="I12" s="10"/>
+      <c r="J12" s="10"/>
+      <c r="K12" s="10" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="42" customHeight="1">
+      <c r="A13" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="H13" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="I13" s="10"/>
+      <c r="J13" s="10"/>
+      <c r="K13" s="10" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="42" customHeight="1">
+      <c r="A14" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="H14" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="I14" s="10"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="10" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="42" customHeight="1">
+      <c r="A15" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="B15" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="G15" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="H15" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10"/>
+      <c r="K15" s="10" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="42" customHeight="1">
+      <c r="A16" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="H16" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="I16" s="10"/>
+      <c r="J16" s="10"/>
+      <c r="K16" s="10" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="42" customHeight="1">
+      <c r="A17" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>188</v>
+      </c>
+      <c r="H17" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="I17" s="10"/>
+      <c r="J17" s="10"/>
+      <c r="K17" s="10" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="42" customHeight="1">
+      <c r="A18" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="C18" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="F6" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="G6" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="H6" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="I6" s="10" t="s">
+      <c r="D18" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="G18" s="10" t="s">
+        <v>190</v>
+      </c>
+      <c r="H18" s="12" t="s">
+        <v>137</v>
+      </c>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="10" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="42" customHeight="1">
+      <c r="A19" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="B19" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="C19" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="J6" s="10" t="s">
-        <v>109</v>
-      </c>
-      <c r="K6" s="10" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="42" customHeight="1">
-      <c r="A7" s="15" t="s">
-        <v>111</v>
-      </c>
-      <c r="B7" s="16" t="s">
-        <v>153</v>
-      </c>
-      <c r="C7" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>196</v>
-      </c>
-      <c r="F7" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="G7" s="12" t="s">
-        <v>210</v>
-      </c>
-      <c r="H7" s="14" t="s">
-        <v>155</v>
-      </c>
-      <c r="I7" s="12"/>
-      <c r="J7" s="12"/>
-      <c r="K7" s="12" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="42" customHeight="1">
-      <c r="A8" s="15" t="s">
-        <v>112</v>
-      </c>
-      <c r="B8" s="16" t="s">
-        <v>153</v>
-      </c>
-      <c r="C8" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="E8" s="11" t="s">
-        <v>196</v>
-      </c>
-      <c r="F8" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="G8" s="12" t="s">
-        <v>212</v>
-      </c>
-      <c r="H8" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="I8" s="12"/>
-      <c r="J8" s="12"/>
-      <c r="K8" s="12" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" ht="42" customHeight="1">
-      <c r="A9" s="15" t="s">
+      <c r="D19" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="B9" s="16" t="s">
-        <v>157</v>
-      </c>
-      <c r="C9" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>196</v>
-      </c>
-      <c r="F9" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="G9" s="12" t="s">
-        <v>214</v>
-      </c>
-      <c r="H9" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="I9" s="12"/>
-      <c r="J9" s="12"/>
-      <c r="K9" s="12" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" ht="42" customHeight="1">
-      <c r="A10" s="15" t="s">
-        <v>114</v>
-      </c>
-      <c r="B10" s="16" t="s">
-        <v>159</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="E10" s="11" t="s">
-        <v>196</v>
-      </c>
-      <c r="F10" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="G10" s="12" t="s">
-        <v>216</v>
-      </c>
-      <c r="H10" s="14" t="s">
-        <v>160</v>
-      </c>
-      <c r="I10" s="12"/>
-      <c r="J10" s="12"/>
-      <c r="K10" s="12" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" ht="42" customHeight="1">
-      <c r="A11" s="15" t="s">
-        <v>115</v>
-      </c>
-      <c r="B11" s="16" t="s">
-        <v>161</v>
-      </c>
-      <c r="C11" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="E11" s="11" t="s">
-        <v>196</v>
-      </c>
-      <c r="F11" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="G11" s="12" t="s">
-        <v>218</v>
-      </c>
-      <c r="H11" s="14" t="s">
-        <v>162</v>
-      </c>
-      <c r="I11" s="12"/>
-      <c r="J11" s="12"/>
-      <c r="K11" s="12" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" ht="42" customHeight="1">
-      <c r="A12" s="15" t="s">
-        <v>116</v>
-      </c>
-      <c r="B12" s="16" t="s">
-        <v>163</v>
-      </c>
-      <c r="C12" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="E12" s="11" t="s">
-        <v>196</v>
-      </c>
-      <c r="F12" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="G12" s="12" t="s">
-        <v>220</v>
-      </c>
-      <c r="H12" s="14" t="s">
-        <v>164</v>
-      </c>
-      <c r="I12" s="12"/>
-      <c r="J12" s="12"/>
-      <c r="K12" s="12" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="42" customHeight="1">
-      <c r="A13" s="15" t="s">
-        <v>117</v>
-      </c>
-      <c r="B13" s="16" t="s">
-        <v>165</v>
-      </c>
-      <c r="C13" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="E13" s="11" t="s">
-        <v>196</v>
-      </c>
-      <c r="F13" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="G13" s="12" t="s">
-        <v>222</v>
-      </c>
-      <c r="H13" s="14" t="s">
-        <v>166</v>
-      </c>
-      <c r="I13" s="12"/>
-      <c r="J13" s="12"/>
-      <c r="K13" s="12" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="42" customHeight="1">
-      <c r="A14" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="B14" s="16" t="s">
-        <v>167</v>
-      </c>
-      <c r="C14" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>196</v>
-      </c>
-      <c r="F14" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="G14" s="12" t="s">
-        <v>224</v>
-      </c>
-      <c r="H14" s="14" t="s">
-        <v>168</v>
-      </c>
-      <c r="I14" s="12"/>
-      <c r="J14" s="12"/>
-      <c r="K14" s="12" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" ht="42" customHeight="1">
-      <c r="A15" s="15" t="s">
-        <v>169</v>
-      </c>
-      <c r="B15" s="16" t="s">
-        <v>170</v>
-      </c>
-      <c r="C15" s="15" t="s">
-        <v>128</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>196</v>
-      </c>
-      <c r="F15" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="G15" s="12" t="s">
-        <v>226</v>
-      </c>
-      <c r="H15" s="14" t="s">
-        <v>171</v>
-      </c>
-      <c r="I15" s="12"/>
-      <c r="J15" s="12"/>
-      <c r="K15" s="12" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" ht="42" customHeight="1">
-      <c r="A16" s="15" t="s">
-        <v>172</v>
-      </c>
-      <c r="B16" s="16" t="s">
-        <v>170</v>
-      </c>
-      <c r="C16" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="D16" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="E16" s="11" t="s">
-        <v>196</v>
-      </c>
-      <c r="F16" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="G16" s="12" t="s">
-        <v>228</v>
-      </c>
-      <c r="H16" s="14" t="s">
-        <v>173</v>
-      </c>
-      <c r="I16" s="12"/>
-      <c r="J16" s="12"/>
-      <c r="K16" s="12" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="42" customHeight="1">
-      <c r="A17" s="15" t="s">
-        <v>174</v>
-      </c>
-      <c r="B17" s="16" t="s">
-        <v>175</v>
-      </c>
-      <c r="C17" s="15" t="s">
-        <v>141</v>
-      </c>
-      <c r="D17" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="E17" s="11" t="s">
-        <v>196</v>
-      </c>
-      <c r="F17" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="G17" s="12" t="s">
-        <v>230</v>
-      </c>
-      <c r="H17" s="14" t="s">
-        <v>176</v>
-      </c>
-      <c r="I17" s="12"/>
-      <c r="J17" s="12"/>
-      <c r="K17" s="12" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" ht="42" customHeight="1">
-      <c r="A18" s="15" t="s">
-        <v>177</v>
-      </c>
-      <c r="B18" s="16" t="s">
-        <v>175</v>
-      </c>
-      <c r="C18" s="15" t="s">
-        <v>145</v>
-      </c>
-      <c r="D18" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="E18" s="11" t="s">
-        <v>196</v>
-      </c>
-      <c r="F18" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="G18" s="12" t="s">
-        <v>232</v>
-      </c>
-      <c r="H18" s="14" t="s">
-        <v>178</v>
-      </c>
-      <c r="I18" s="12"/>
-      <c r="J18" s="12"/>
-      <c r="K18" s="12" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" ht="42" customHeight="1">
-      <c r="A19" s="15" t="s">
-        <v>179</v>
-      </c>
-      <c r="B19" s="16" t="s">
-        <v>180</v>
-      </c>
-      <c r="C19" s="15" t="s">
-        <v>149</v>
-      </c>
-      <c r="D19" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="E19" s="11" t="s">
-        <v>196</v>
-      </c>
-      <c r="F19" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="G19" s="12" t="s">
-        <v>234</v>
-      </c>
-      <c r="H19" s="14" t="s">
-        <v>181</v>
-      </c>
-      <c r="I19" s="12"/>
-      <c r="J19" s="12"/>
-      <c r="K19" s="12" t="s">
-        <v>235</v>
+      <c r="E19" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="G19" s="10" t="s">
+        <v>192</v>
+      </c>
+      <c r="H19" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="10" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="36" customHeight="1">
-      <c r="A20" s="15"/>
-      <c r="B20" s="16"/>
-      <c r="C20" s="15"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="13"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="12"/>
-      <c r="J20" s="12"/>
-      <c r="K20" s="12"/>
+      <c r="A20" s="13"/>
+      <c r="B20" s="14"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="12"/>
+      <c r="I20" s="10"/>
+      <c r="J20" s="10"/>
+      <c r="K20" s="10"/>
     </row>
     <row r="21" spans="1:11" ht="36" customHeight="1">
-      <c r="A21" s="15"/>
-      <c r="B21" s="16"/>
-      <c r="C21" s="15"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="12"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="12"/>
-      <c r="J21" s="12"/>
-      <c r="K21" s="12"/>
+      <c r="A21" s="13"/>
+      <c r="B21" s="14"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="12"/>
+      <c r="I21" s="10"/>
+      <c r="J21" s="10"/>
+      <c r="K21" s="10"/>
     </row>
     <row r="22" spans="1:11" ht="36" customHeight="1">
-      <c r="A22" s="15"/>
-      <c r="B22" s="16"/>
-      <c r="C22" s="15"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="13"/>
-      <c r="G22" s="12"/>
-      <c r="H22" s="14"/>
-      <c r="I22" s="12"/>
-      <c r="J22" s="12"/>
-      <c r="K22" s="12"/>
+      <c r="A22" s="13"/>
+      <c r="B22" s="14"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="10"/>
+      <c r="H22" s="12"/>
+      <c r="I22" s="10"/>
+      <c r="J22" s="10"/>
+      <c r="K22" s="10"/>
     </row>
     <row r="23" spans="1:11" ht="36" customHeight="1">
-      <c r="A23" s="15"/>
-      <c r="B23" s="16"/>
-      <c r="C23" s="15"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="13"/>
-      <c r="G23" s="12"/>
-      <c r="H23" s="14"/>
-      <c r="I23" s="12"/>
-      <c r="J23" s="12"/>
-      <c r="K23" s="12"/>
+      <c r="A23" s="13"/>
+      <c r="B23" s="14"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="11"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="12"/>
+      <c r="I23" s="10"/>
+      <c r="J23" s="10"/>
+      <c r="K23" s="10"/>
     </row>
     <row r="24" spans="1:11" ht="36" customHeight="1">
-      <c r="A24" s="15"/>
-      <c r="B24" s="16"/>
-      <c r="C24" s="15"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="12"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="12"/>
-      <c r="J24" s="12"/>
-      <c r="K24" s="12"/>
+      <c r="A24" s="13"/>
+      <c r="B24" s="14"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="11"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="12"/>
+      <c r="I24" s="10"/>
+      <c r="J24" s="10"/>
+      <c r="K24" s="10"/>
     </row>
     <row r="25" spans="1:11" ht="36" customHeight="1">
-      <c r="A25" s="15"/>
-      <c r="B25" s="16"/>
-      <c r="C25" s="15"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
-      <c r="F25" s="13"/>
-      <c r="G25" s="12"/>
-      <c r="H25" s="14"/>
-      <c r="I25" s="12"/>
-      <c r="J25" s="12"/>
-      <c r="K25" s="12"/>
+      <c r="A25" s="13"/>
+      <c r="B25" s="14"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="11"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="12"/>
+      <c r="I25" s="10"/>
+      <c r="J25" s="10"/>
+      <c r="K25" s="10"/>
     </row>
     <row r="26" spans="1:11" ht="36" customHeight="1">
-      <c r="A26" s="15"/>
-      <c r="B26" s="16"/>
-      <c r="C26" s="15"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
-      <c r="F26" s="13"/>
-      <c r="G26" s="12"/>
-      <c r="H26" s="14"/>
-      <c r="I26" s="12"/>
-      <c r="J26" s="12"/>
-      <c r="K26" s="12"/>
+      <c r="A26" s="13"/>
+      <c r="B26" s="14"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="11"/>
+      <c r="G26" s="10"/>
+      <c r="H26" s="12"/>
+      <c r="I26" s="10"/>
+      <c r="J26" s="10"/>
+      <c r="K26" s="10"/>
     </row>
     <row r="27" spans="1:11" ht="36" customHeight="1">
-      <c r="A27" s="15"/>
-      <c r="B27" s="16"/>
-      <c r="C27" s="15"/>
-      <c r="D27" s="11"/>
-      <c r="E27" s="11"/>
-      <c r="F27" s="13"/>
-      <c r="G27" s="12"/>
-      <c r="H27" s="14"/>
-      <c r="I27" s="12"/>
-      <c r="J27" s="12"/>
-      <c r="K27" s="12"/>
+      <c r="A27" s="13"/>
+      <c r="B27" s="14"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="11"/>
+      <c r="G27" s="10"/>
+      <c r="H27" s="12"/>
+      <c r="I27" s="10"/>
+      <c r="J27" s="10"/>
+      <c r="K27" s="10"/>
     </row>
     <row r="28" spans="1:11" ht="36" customHeight="1">
-      <c r="A28" s="15"/>
-      <c r="B28" s="16"/>
-      <c r="C28" s="15"/>
-      <c r="D28" s="11"/>
-      <c r="E28" s="11"/>
-      <c r="F28" s="13"/>
-      <c r="G28" s="12"/>
-      <c r="H28" s="14"/>
-      <c r="I28" s="12"/>
-      <c r="J28" s="12"/>
-      <c r="K28" s="12"/>
+      <c r="A28" s="13"/>
+      <c r="B28" s="14"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="9"/>
+      <c r="E28" s="9"/>
+      <c r="F28" s="11"/>
+      <c r="G28" s="10"/>
+      <c r="H28" s="12"/>
+      <c r="I28" s="10"/>
+      <c r="J28" s="10"/>
+      <c r="K28" s="10"/>
     </row>
     <row r="29" spans="1:11" ht="36" customHeight="1">
-      <c r="A29" s="15"/>
-      <c r="B29" s="16"/>
-      <c r="C29" s="15"/>
-      <c r="D29" s="11"/>
-      <c r="E29" s="11"/>
-      <c r="F29" s="13"/>
-      <c r="G29" s="12"/>
-      <c r="H29" s="14"/>
-      <c r="I29" s="12"/>
-      <c r="J29" s="12"/>
-      <c r="K29" s="12"/>
+      <c r="A29" s="13"/>
+      <c r="B29" s="14"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="9"/>
+      <c r="E29" s="9"/>
+      <c r="F29" s="11"/>
+      <c r="G29" s="10"/>
+      <c r="H29" s="12"/>
+      <c r="I29" s="10"/>
+      <c r="J29" s="10"/>
+      <c r="K29" s="10"/>
     </row>
     <row r="30" spans="1:11" ht="36" customHeight="1">
-      <c r="A30" s="15"/>
-      <c r="B30" s="16"/>
-      <c r="C30" s="15"/>
-      <c r="D30" s="11"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="13"/>
-      <c r="G30" s="12"/>
-      <c r="H30" s="14"/>
-      <c r="I30" s="12"/>
-      <c r="J30" s="12"/>
-      <c r="K30" s="12"/>
+      <c r="A30" s="13"/>
+      <c r="B30" s="14"/>
+      <c r="C30" s="13"/>
+      <c r="D30" s="9"/>
+      <c r="E30" s="9"/>
+      <c r="F30" s="11"/>
+      <c r="G30" s="10"/>
+      <c r="H30" s="12"/>
+      <c r="I30" s="10"/>
+      <c r="J30" s="10"/>
+      <c r="K30" s="10"/>
     </row>
     <row r="31" spans="1:11" ht="36" customHeight="1">
-      <c r="A31" s="15"/>
-      <c r="B31" s="16"/>
-      <c r="C31" s="15"/>
-      <c r="D31" s="11"/>
-      <c r="E31" s="11"/>
-      <c r="F31" s="13"/>
-      <c r="G31" s="12"/>
-      <c r="H31" s="14"/>
-      <c r="I31" s="12"/>
-      <c r="J31" s="12"/>
-      <c r="K31" s="12"/>
+      <c r="A31" s="13"/>
+      <c r="B31" s="14"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="9"/>
+      <c r="E31" s="9"/>
+      <c r="F31" s="11"/>
+      <c r="G31" s="10"/>
+      <c r="H31" s="12"/>
+      <c r="I31" s="10"/>
+      <c r="J31" s="10"/>
+      <c r="K31" s="10"/>
     </row>
     <row r="32" spans="1:11" ht="36" customHeight="1">
-      <c r="A32" s="15"/>
-      <c r="B32" s="16"/>
-      <c r="C32" s="15"/>
-      <c r="D32" s="11"/>
-      <c r="E32" s="11"/>
-      <c r="F32" s="13"/>
-      <c r="G32" s="12"/>
-      <c r="H32" s="14"/>
-      <c r="I32" s="12"/>
-      <c r="J32" s="12"/>
-      <c r="K32" s="12"/>
+      <c r="A32" s="13"/>
+      <c r="B32" s="14"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="9"/>
+      <c r="F32" s="11"/>
+      <c r="G32" s="10"/>
+      <c r="H32" s="12"/>
+      <c r="I32" s="10"/>
+      <c r="J32" s="10"/>
+      <c r="K32" s="10"/>
     </row>
     <row r="33" spans="1:11" ht="36" customHeight="1">
-      <c r="A33" s="15"/>
-      <c r="B33" s="16"/>
-      <c r="C33" s="15"/>
-      <c r="D33" s="11"/>
-      <c r="E33" s="11"/>
-      <c r="F33" s="13"/>
-      <c r="G33" s="12"/>
-      <c r="H33" s="14"/>
-      <c r="I33" s="12"/>
-      <c r="J33" s="12"/>
-      <c r="K33" s="12"/>
+      <c r="A33" s="13"/>
+      <c r="B33" s="14"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="11"/>
+      <c r="G33" s="10"/>
+      <c r="H33" s="12"/>
+      <c r="I33" s="10"/>
+      <c r="J33" s="10"/>
+      <c r="K33" s="10"/>
     </row>
     <row r="34" spans="1:11" ht="36" customHeight="1">
-      <c r="A34" s="15"/>
-      <c r="B34" s="16"/>
-      <c r="C34" s="15"/>
-      <c r="D34" s="11"/>
-      <c r="E34" s="11"/>
-      <c r="F34" s="13"/>
-      <c r="G34" s="12"/>
-      <c r="H34" s="14"/>
-      <c r="I34" s="12"/>
-      <c r="J34" s="12"/>
-      <c r="K34" s="12"/>
+      <c r="A34" s="13"/>
+      <c r="B34" s="14"/>
+      <c r="C34" s="13"/>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="11"/>
+      <c r="G34" s="10"/>
+      <c r="H34" s="12"/>
+      <c r="I34" s="10"/>
+      <c r="J34" s="10"/>
+      <c r="K34" s="10"/>
     </row>
     <row r="35" spans="1:11" ht="36" customHeight="1">
-      <c r="A35" s="15"/>
-      <c r="B35" s="16"/>
-      <c r="C35" s="15"/>
-      <c r="D35" s="11"/>
-      <c r="E35" s="11"/>
-      <c r="F35" s="13"/>
-      <c r="G35" s="12"/>
-      <c r="H35" s="14"/>
-      <c r="I35" s="12"/>
-      <c r="J35" s="12"/>
-      <c r="K35" s="12"/>
+      <c r="A35" s="13"/>
+      <c r="B35" s="14"/>
+      <c r="C35" s="13"/>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="11"/>
+      <c r="G35" s="10"/>
+      <c r="H35" s="12"/>
+      <c r="I35" s="10"/>
+      <c r="J35" s="10"/>
+      <c r="K35" s="10"/>
     </row>
     <row r="36" spans="1:11" ht="36" customHeight="1">
-      <c r="A36" s="15"/>
-      <c r="B36" s="16"/>
-      <c r="C36" s="15"/>
-      <c r="D36" s="11"/>
-      <c r="E36" s="11"/>
-      <c r="F36" s="13"/>
-      <c r="G36" s="12"/>
-      <c r="H36" s="14"/>
-      <c r="I36" s="12"/>
-      <c r="J36" s="12"/>
-      <c r="K36" s="12"/>
+      <c r="A36" s="13"/>
+      <c r="B36" s="14"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="11"/>
+      <c r="G36" s="10"/>
+      <c r="H36" s="12"/>
+      <c r="I36" s="10"/>
+      <c r="J36" s="10"/>
+      <c r="K36" s="10"/>
     </row>
     <row r="37" spans="1:11" ht="36" customHeight="1">
-      <c r="A37" s="15"/>
-      <c r="B37" s="16"/>
-      <c r="C37" s="15"/>
-      <c r="D37" s="11"/>
-      <c r="E37" s="11"/>
-      <c r="F37" s="13"/>
-      <c r="G37" s="12"/>
-      <c r="H37" s="14"/>
-      <c r="I37" s="12"/>
-      <c r="J37" s="12"/>
-      <c r="K37" s="12"/>
+      <c r="A37" s="13"/>
+      <c r="B37" s="14"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="9"/>
+      <c r="E37" s="9"/>
+      <c r="F37" s="11"/>
+      <c r="G37" s="10"/>
+      <c r="H37" s="12"/>
+      <c r="I37" s="10"/>
+      <c r="J37" s="10"/>
+      <c r="K37" s="10"/>
     </row>
     <row r="38" spans="1:11" ht="36" customHeight="1">
-      <c r="A38" s="15"/>
-      <c r="B38" s="16"/>
-      <c r="C38" s="15"/>
-      <c r="D38" s="11"/>
-      <c r="E38" s="11"/>
-      <c r="F38" s="13"/>
-      <c r="G38" s="12"/>
-      <c r="H38" s="14"/>
-      <c r="I38" s="12"/>
-      <c r="J38" s="12"/>
-      <c r="K38" s="12"/>
+      <c r="A38" s="13"/>
+      <c r="B38" s="14"/>
+      <c r="C38" s="13"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="9"/>
+      <c r="F38" s="11"/>
+      <c r="G38" s="10"/>
+      <c r="H38" s="12"/>
+      <c r="I38" s="10"/>
+      <c r="J38" s="10"/>
+      <c r="K38" s="10"/>
     </row>
     <row r="39" spans="1:11" ht="36" customHeight="1">
-      <c r="A39" s="15"/>
-      <c r="B39" s="16"/>
-      <c r="C39" s="15"/>
-      <c r="D39" s="11"/>
-      <c r="E39" s="11"/>
-      <c r="F39" s="13"/>
-      <c r="G39" s="12"/>
-      <c r="H39" s="14"/>
-      <c r="I39" s="12"/>
-      <c r="J39" s="12"/>
-      <c r="K39" s="12"/>
+      <c r="A39" s="13"/>
+      <c r="B39" s="14"/>
+      <c r="C39" s="13"/>
+      <c r="D39" s="9"/>
+      <c r="E39" s="9"/>
+      <c r="F39" s="11"/>
+      <c r="G39" s="10"/>
+      <c r="H39" s="12"/>
+      <c r="I39" s="10"/>
+      <c r="J39" s="10"/>
+      <c r="K39" s="10"/>
     </row>
     <row r="40" spans="1:11" ht="36" customHeight="1">
-      <c r="A40" s="15"/>
-      <c r="B40" s="16"/>
-      <c r="C40" s="15"/>
-      <c r="D40" s="11"/>
-      <c r="E40" s="11"/>
-      <c r="F40" s="13"/>
-      <c r="G40" s="12"/>
-      <c r="H40" s="14"/>
-      <c r="I40" s="12"/>
-      <c r="J40" s="12"/>
-      <c r="K40" s="12"/>
+      <c r="A40" s="13"/>
+      <c r="B40" s="14"/>
+      <c r="C40" s="13"/>
+      <c r="D40" s="9"/>
+      <c r="E40" s="9"/>
+      <c r="F40" s="11"/>
+      <c r="G40" s="10"/>
+      <c r="H40" s="12"/>
+      <c r="I40" s="10"/>
+      <c r="J40" s="10"/>
+      <c r="K40" s="10"/>
     </row>
     <row r="41" spans="1:11" ht="36" customHeight="1">
-      <c r="A41" s="15"/>
-      <c r="B41" s="16"/>
-      <c r="C41" s="15"/>
-      <c r="D41" s="11"/>
-      <c r="E41" s="11"/>
-      <c r="F41" s="13"/>
-      <c r="G41" s="12"/>
-      <c r="H41" s="14"/>
-      <c r="I41" s="12"/>
-      <c r="J41" s="12"/>
-      <c r="K41" s="12"/>
+      <c r="A41" s="13"/>
+      <c r="B41" s="14"/>
+      <c r="C41" s="13"/>
+      <c r="D41" s="9"/>
+      <c r="E41" s="9"/>
+      <c r="F41" s="11"/>
+      <c r="G41" s="10"/>
+      <c r="H41" s="12"/>
+      <c r="I41" s="10"/>
+      <c r="J41" s="10"/>
+      <c r="K41" s="10"/>
     </row>
     <row r="42" spans="1:11" ht="36" customHeight="1">
-      <c r="A42" s="15"/>
-      <c r="B42" s="16"/>
-      <c r="C42" s="15"/>
-      <c r="D42" s="11"/>
-      <c r="E42" s="11"/>
-      <c r="F42" s="13"/>
-      <c r="G42" s="12"/>
-      <c r="H42" s="14"/>
-      <c r="I42" s="12"/>
-      <c r="J42" s="12"/>
-      <c r="K42" s="12"/>
+      <c r="A42" s="13"/>
+      <c r="B42" s="14"/>
+      <c r="C42" s="13"/>
+      <c r="D42" s="9"/>
+      <c r="E42" s="9"/>
+      <c r="F42" s="11"/>
+      <c r="G42" s="10"/>
+      <c r="H42" s="12"/>
+      <c r="I42" s="10"/>
+      <c r="J42" s="10"/>
+      <c r="K42" s="10"/>
     </row>
     <row r="43" spans="1:11" ht="36" customHeight="1">
-      <c r="A43" s="15"/>
-      <c r="B43" s="16"/>
-      <c r="C43" s="15"/>
-      <c r="D43" s="11"/>
-      <c r="E43" s="11"/>
-      <c r="F43" s="13"/>
-      <c r="G43" s="12"/>
-      <c r="H43" s="14"/>
-      <c r="I43" s="12"/>
-      <c r="J43" s="12"/>
-      <c r="K43" s="12"/>
+      <c r="A43" s="13"/>
+      <c r="B43" s="14"/>
+      <c r="C43" s="13"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="9"/>
+      <c r="F43" s="11"/>
+      <c r="G43" s="10"/>
+      <c r="H43" s="12"/>
+      <c r="I43" s="10"/>
+      <c r="J43" s="10"/>
+      <c r="K43" s="10"/>
     </row>
     <row r="44" spans="1:11" ht="36" customHeight="1">
-      <c r="A44" s="15"/>
-      <c r="B44" s="16"/>
-      <c r="C44" s="15"/>
-      <c r="D44" s="11"/>
-      <c r="E44" s="11"/>
-      <c r="F44" s="13"/>
-      <c r="G44" s="12"/>
-      <c r="H44" s="14"/>
-      <c r="I44" s="12"/>
-      <c r="J44" s="12"/>
-      <c r="K44" s="12"/>
+      <c r="A44" s="13"/>
+      <c r="B44" s="14"/>
+      <c r="C44" s="13"/>
+      <c r="D44" s="9"/>
+      <c r="E44" s="9"/>
+      <c r="F44" s="11"/>
+      <c r="G44" s="10"/>
+      <c r="H44" s="12"/>
+      <c r="I44" s="10"/>
+      <c r="J44" s="10"/>
+      <c r="K44" s="10"/>
     </row>
     <row r="45" spans="1:11" ht="36" customHeight="1">
-      <c r="A45" s="15"/>
-      <c r="B45" s="16"/>
-      <c r="C45" s="15"/>
-      <c r="D45" s="11"/>
-      <c r="E45" s="11"/>
-      <c r="F45" s="13"/>
-      <c r="G45" s="12"/>
-      <c r="H45" s="14"/>
-      <c r="I45" s="12"/>
-      <c r="J45" s="12"/>
-      <c r="K45" s="12"/>
+      <c r="A45" s="13"/>
+      <c r="B45" s="14"/>
+      <c r="C45" s="13"/>
+      <c r="D45" s="9"/>
+      <c r="E45" s="9"/>
+      <c r="F45" s="11"/>
+      <c r="G45" s="10"/>
+      <c r="H45" s="12"/>
+      <c r="I45" s="10"/>
+      <c r="J45" s="10"/>
+      <c r="K45" s="10"/>
     </row>
     <row r="46" spans="1:11" ht="36" customHeight="1">
-      <c r="A46" s="15"/>
-      <c r="B46" s="16"/>
-      <c r="C46" s="15"/>
-      <c r="D46" s="11"/>
-      <c r="E46" s="11"/>
-      <c r="F46" s="13"/>
-      <c r="G46" s="12"/>
-      <c r="H46" s="14"/>
-      <c r="I46" s="12"/>
-      <c r="J46" s="12"/>
-      <c r="K46" s="12"/>
+      <c r="A46" s="13"/>
+      <c r="B46" s="14"/>
+      <c r="C46" s="13"/>
+      <c r="D46" s="9"/>
+      <c r="E46" s="9"/>
+      <c r="F46" s="11"/>
+      <c r="G46" s="10"/>
+      <c r="H46" s="12"/>
+      <c r="I46" s="10"/>
+      <c r="J46" s="10"/>
+      <c r="K46" s="10"/>
     </row>
     <row r="47" spans="1:11" ht="36" customHeight="1">
-      <c r="A47" s="15"/>
-      <c r="B47" s="16"/>
-      <c r="C47" s="15"/>
-      <c r="D47" s="11"/>
-      <c r="E47" s="11"/>
-      <c r="F47" s="13"/>
-      <c r="G47" s="12"/>
-      <c r="H47" s="14"/>
-      <c r="I47" s="12"/>
-      <c r="J47" s="12"/>
-      <c r="K47" s="12"/>
+      <c r="A47" s="13"/>
+      <c r="B47" s="14"/>
+      <c r="C47" s="13"/>
+      <c r="D47" s="9"/>
+      <c r="E47" s="9"/>
+      <c r="F47" s="11"/>
+      <c r="G47" s="10"/>
+      <c r="H47" s="12"/>
+      <c r="I47" s="10"/>
+      <c r="J47" s="10"/>
+      <c r="K47" s="10"/>
     </row>
     <row r="48" spans="1:11" ht="36" customHeight="1">
-      <c r="A48" s="15"/>
-      <c r="B48" s="16"/>
-      <c r="C48" s="15"/>
-      <c r="D48" s="11"/>
-      <c r="E48" s="11"/>
-      <c r="F48" s="13"/>
-      <c r="G48" s="12"/>
-      <c r="H48" s="14"/>
-      <c r="I48" s="12"/>
-      <c r="J48" s="12"/>
-      <c r="K48" s="12"/>
+      <c r="A48" s="13"/>
+      <c r="B48" s="14"/>
+      <c r="C48" s="13"/>
+      <c r="D48" s="9"/>
+      <c r="E48" s="9"/>
+      <c r="F48" s="11"/>
+      <c r="G48" s="10"/>
+      <c r="H48" s="12"/>
+      <c r="I48" s="10"/>
+      <c r="J48" s="10"/>
+      <c r="K48" s="10"/>
     </row>
     <row r="49" spans="1:11" ht="36" customHeight="1">
-      <c r="A49" s="15"/>
-      <c r="B49" s="16"/>
-      <c r="C49" s="15"/>
-      <c r="D49" s="11"/>
-      <c r="E49" s="11"/>
-      <c r="F49" s="13"/>
-      <c r="G49" s="12"/>
-      <c r="H49" s="14"/>
-      <c r="I49" s="12"/>
-      <c r="J49" s="12"/>
-      <c r="K49" s="12"/>
+      <c r="A49" s="13"/>
+      <c r="B49" s="14"/>
+      <c r="C49" s="13"/>
+      <c r="D49" s="9"/>
+      <c r="E49" s="9"/>
+      <c r="F49" s="11"/>
+      <c r="G49" s="10"/>
+      <c r="H49" s="12"/>
+      <c r="I49" s="10"/>
+      <c r="J49" s="10"/>
+      <c r="K49" s="10"/>
     </row>
     <row r="50" spans="1:11" ht="36" customHeight="1">
-      <c r="A50" s="15"/>
-      <c r="B50" s="16"/>
-      <c r="C50" s="15"/>
-      <c r="D50" s="11"/>
-      <c r="E50" s="11"/>
-      <c r="F50" s="13"/>
-      <c r="G50" s="12"/>
-      <c r="H50" s="14"/>
-      <c r="I50" s="12"/>
-      <c r="J50" s="12"/>
-      <c r="K50" s="12"/>
+      <c r="A50" s="13"/>
+      <c r="B50" s="14"/>
+      <c r="C50" s="13"/>
+      <c r="D50" s="9"/>
+      <c r="E50" s="9"/>
+      <c r="F50" s="11"/>
+      <c r="G50" s="10"/>
+      <c r="H50" s="12"/>
+      <c r="I50" s="10"/>
+      <c r="J50" s="10"/>
+      <c r="K50" s="10"/>
     </row>
     <row r="51" spans="1:11" ht="36" customHeight="1">
-      <c r="A51" s="15"/>
-      <c r="B51" s="16"/>
-      <c r="C51" s="15"/>
-      <c r="D51" s="11"/>
-      <c r="E51" s="11"/>
-      <c r="F51" s="13"/>
-      <c r="G51" s="12"/>
-      <c r="H51" s="14"/>
-      <c r="I51" s="12"/>
-      <c r="J51" s="12"/>
-      <c r="K51" s="12"/>
+      <c r="A51" s="13"/>
+      <c r="B51" s="14"/>
+      <c r="C51" s="13"/>
+      <c r="D51" s="9"/>
+      <c r="E51" s="9"/>
+      <c r="F51" s="11"/>
+      <c r="G51" s="10"/>
+      <c r="H51" s="12"/>
+      <c r="I51" s="10"/>
+      <c r="J51" s="10"/>
+      <c r="K51" s="10"/>
     </row>
     <row r="52" spans="1:11" ht="36" customHeight="1">
-      <c r="A52" s="15"/>
-      <c r="B52" s="16"/>
-      <c r="C52" s="15"/>
-      <c r="D52" s="11"/>
-      <c r="E52" s="11"/>
-      <c r="F52" s="13"/>
-      <c r="G52" s="12"/>
-      <c r="H52" s="14"/>
-      <c r="I52" s="12"/>
-      <c r="J52" s="12"/>
-      <c r="K52" s="12"/>
+      <c r="A52" s="13"/>
+      <c r="B52" s="14"/>
+      <c r="C52" s="13"/>
+      <c r="D52" s="9"/>
+      <c r="E52" s="9"/>
+      <c r="F52" s="11"/>
+      <c r="G52" s="10"/>
+      <c r="H52" s="12"/>
+      <c r="I52" s="10"/>
+      <c r="J52" s="10"/>
+      <c r="K52" s="10"/>
     </row>
     <row r="53" spans="1:11" ht="36" customHeight="1">
-      <c r="A53" s="15"/>
-      <c r="B53" s="16"/>
-      <c r="C53" s="15"/>
-      <c r="D53" s="11"/>
-      <c r="E53" s="11"/>
-      <c r="F53" s="13"/>
-      <c r="G53" s="12"/>
-      <c r="H53" s="14"/>
-      <c r="I53" s="12"/>
-      <c r="J53" s="12"/>
-      <c r="K53" s="12"/>
+      <c r="A53" s="13"/>
+      <c r="B53" s="14"/>
+      <c r="C53" s="13"/>
+      <c r="D53" s="9"/>
+      <c r="E53" s="9"/>
+      <c r="F53" s="11"/>
+      <c r="G53" s="10"/>
+      <c r="H53" s="12"/>
+      <c r="I53" s="10"/>
+      <c r="J53" s="10"/>
+      <c r="K53" s="10"/>
     </row>
     <row r="54" spans="1:11" ht="36" customHeight="1">
-      <c r="A54" s="15"/>
-      <c r="B54" s="16"/>
-      <c r="C54" s="15"/>
-      <c r="D54" s="11"/>
-      <c r="E54" s="11"/>
-      <c r="F54" s="13"/>
-      <c r="G54" s="12"/>
-      <c r="H54" s="14"/>
-      <c r="I54" s="12"/>
-      <c r="J54" s="12"/>
-      <c r="K54" s="12"/>
+      <c r="A54" s="13"/>
+      <c r="B54" s="14"/>
+      <c r="C54" s="13"/>
+      <c r="D54" s="9"/>
+      <c r="E54" s="9"/>
+      <c r="F54" s="11"/>
+      <c r="G54" s="10"/>
+      <c r="H54" s="12"/>
+      <c r="I54" s="10"/>
+      <c r="J54" s="10"/>
+      <c r="K54" s="10"/>
     </row>
     <row r="55" spans="1:11" ht="36" customHeight="1">
-      <c r="A55" s="15"/>
-      <c r="B55" s="16"/>
-      <c r="C55" s="15"/>
-      <c r="D55" s="11"/>
-      <c r="E55" s="11"/>
-      <c r="F55" s="13"/>
-      <c r="G55" s="12"/>
-      <c r="H55" s="14"/>
-      <c r="I55" s="12"/>
-      <c r="J55" s="12"/>
-      <c r="K55" s="12"/>
+      <c r="A55" s="13"/>
+      <c r="B55" s="14"/>
+      <c r="C55" s="13"/>
+      <c r="D55" s="9"/>
+      <c r="E55" s="9"/>
+      <c r="F55" s="11"/>
+      <c r="G55" s="10"/>
+      <c r="H55" s="12"/>
+      <c r="I55" s="10"/>
+      <c r="J55" s="10"/>
+      <c r="K55" s="10"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F7:F55 G56:G500">
@@ -4885,7 +3879,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <tabColor rgb="FF7892A5"/>
@@ -4916,7 +3910,7 @@
     </row>
     <row r="2" spans="1:12" ht="29.1" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>119</v>
+        <v>81</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -4932,7 +3926,7 @@
     </row>
     <row r="3" spans="1:12" ht="24" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>120</v>
+        <v>82</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -4975,23 +3969,23 @@
       <c r="L5" s="1"/>
     </row>
     <row r="6" spans="1:12" ht="33.950000000000003" customHeight="1">
-      <c r="A6" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="C6" s="10" t="s">
+      <c r="A6" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="10" t="s">
-        <v>122</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="F6" s="10" t="s">
-        <v>124</v>
+      <c r="D6" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>86</v>
       </c>
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
@@ -5001,22 +3995,22 @@
       <c r="L6" s="1"/>
     </row>
     <row r="7" spans="1:12" ht="140.1" customHeight="1">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="D7" s="10" t="s">
         <v>155</v>
       </c>
-      <c r="B7" s="11" t="s">
-        <v>111</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>197</v>
-      </c>
-      <c r="E7" s="20" t="s">
-        <v>183</v>
-      </c>
-      <c r="F7" s="17"/>
+      <c r="E7" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="F7" s="15"/>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
@@ -5025,22 +4019,22 @@
       <c r="L7" s="1"/>
     </row>
     <row r="8" spans="1:12" ht="140.1" customHeight="1">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="D8" s="10" t="s">
         <v>156</v>
       </c>
-      <c r="B8" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="D8" s="12" t="s">
-        <v>198</v>
-      </c>
-      <c r="E8" s="20" t="s">
-        <v>184</v>
-      </c>
-      <c r="F8" s="17"/>
+      <c r="E8" s="18" t="s">
+        <v>143</v>
+      </c>
+      <c r="F8" s="15"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
@@ -5049,22 +4043,22 @@
       <c r="L8" s="1"/>
     </row>
     <row r="9" spans="1:12" ht="140.1" customHeight="1">
-      <c r="A9" s="11" t="s">
-        <v>158</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>113</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="D9" s="12" t="s">
-        <v>199</v>
-      </c>
-      <c r="E9" s="20" t="s">
-        <v>185</v>
-      </c>
-      <c r="F9" s="17"/>
+      <c r="A9" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="E9" s="18" t="s">
+        <v>144</v>
+      </c>
+      <c r="F9" s="15"/>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
@@ -5073,22 +4067,22 @@
       <c r="L9" s="1"/>
     </row>
     <row r="10" spans="1:12" ht="140.1" customHeight="1">
-      <c r="A10" s="11" t="s">
-        <v>160</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="C10" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="D10" s="12" t="s">
-        <v>200</v>
-      </c>
-      <c r="E10" s="20" t="s">
-        <v>186</v>
-      </c>
-      <c r="F10" s="17"/>
+      <c r="A10" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="E10" s="18" t="s">
+        <v>145</v>
+      </c>
+      <c r="F10" s="15"/>
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
@@ -5097,22 +4091,22 @@
       <c r="L10" s="1"/>
     </row>
     <row r="11" spans="1:12" ht="140.1" customHeight="1">
-      <c r="A11" s="11" t="s">
-        <v>162</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="C11" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="D11" s="12" t="s">
-        <v>201</v>
-      </c>
-      <c r="E11" s="20" t="s">
-        <v>187</v>
-      </c>
-      <c r="F11" s="17"/>
+      <c r="A11" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="E11" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="F11" s="15"/>
       <c r="G11" s="1"/>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
@@ -5121,22 +4115,22 @@
       <c r="L11" s="1"/>
     </row>
     <row r="12" spans="1:12" ht="140.1" customHeight="1">
-      <c r="A12" s="11" t="s">
-        <v>164</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="C12" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="D12" s="12" t="s">
-        <v>202</v>
-      </c>
-      <c r="E12" s="20" t="s">
-        <v>188</v>
-      </c>
-      <c r="F12" s="17"/>
+      <c r="A12" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="E12" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="F12" s="15"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
@@ -5145,22 +4139,22 @@
       <c r="L12" s="1"/>
     </row>
     <row r="13" spans="1:12" ht="140.1" customHeight="1">
-      <c r="A13" s="11" t="s">
-        <v>166</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="C13" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="D13" s="12" t="s">
-        <v>203</v>
-      </c>
-      <c r="E13" s="20" t="s">
-        <v>189</v>
-      </c>
-      <c r="F13" s="17"/>
+      <c r="A13" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="E13" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="F13" s="15"/>
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
@@ -5169,22 +4163,22 @@
       <c r="L13" s="1"/>
     </row>
     <row r="14" spans="1:12" ht="140.1" customHeight="1">
-      <c r="A14" s="11" t="s">
-        <v>168</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="D14" s="12" t="s">
-        <v>204</v>
-      </c>
-      <c r="E14" s="20" t="s">
-        <v>190</v>
-      </c>
-      <c r="F14" s="17"/>
+      <c r="A14" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="E14" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="F14" s="15"/>
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
       <c r="I14" s="1"/>
@@ -5193,22 +4187,22 @@
       <c r="L14" s="1"/>
     </row>
     <row r="15" spans="1:12" ht="140.1" customHeight="1">
-      <c r="A15" s="11" t="s">
-        <v>171</v>
-      </c>
-      <c r="B15" s="11" t="s">
-        <v>169</v>
-      </c>
-      <c r="C15" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="D15" s="12" t="s">
-        <v>205</v>
-      </c>
-      <c r="E15" s="20" t="s">
-        <v>191</v>
-      </c>
-      <c r="F15" s="17"/>
+      <c r="A15" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="E15" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="F15" s="15"/>
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
@@ -5217,22 +4211,22 @@
       <c r="L15" s="1"/>
     </row>
     <row r="16" spans="1:12" ht="140.1" customHeight="1">
-      <c r="A16" s="11" t="s">
-        <v>173</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>172</v>
-      </c>
-      <c r="C16" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="D16" s="12" t="s">
-        <v>206</v>
-      </c>
-      <c r="E16" s="20" t="s">
-        <v>192</v>
-      </c>
-      <c r="F16" s="17"/>
+      <c r="A16" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="E16" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="F16" s="15"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
@@ -5241,22 +4235,22 @@
       <c r="L16" s="1"/>
     </row>
     <row r="17" spans="1:12" ht="140.1" customHeight="1">
-      <c r="A17" s="11" t="s">
-        <v>176</v>
-      </c>
-      <c r="B17" s="11" t="s">
-        <v>174</v>
-      </c>
-      <c r="C17" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="D17" s="12" t="s">
-        <v>207</v>
-      </c>
-      <c r="E17" s="20" t="s">
-        <v>193</v>
-      </c>
-      <c r="F17" s="17"/>
+      <c r="A17" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="E17" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="F17" s="15"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
@@ -5265,22 +4259,22 @@
       <c r="L17" s="1"/>
     </row>
     <row r="18" spans="1:12" ht="140.1" customHeight="1">
-      <c r="A18" s="11" t="s">
-        <v>178</v>
-      </c>
-      <c r="B18" s="11" t="s">
-        <v>177</v>
-      </c>
-      <c r="C18" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="D18" s="12" t="s">
-        <v>208</v>
-      </c>
-      <c r="E18" s="20" t="s">
-        <v>194</v>
-      </c>
-      <c r="F18" s="17"/>
+      <c r="A18" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="E18" s="18" t="s">
+        <v>153</v>
+      </c>
+      <c r="F18" s="15"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
@@ -5289,22 +4283,22 @@
       <c r="L18" s="1"/>
     </row>
     <row r="19" spans="1:12" ht="140.1" customHeight="1">
-      <c r="A19" s="11" t="s">
-        <v>181</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>179</v>
-      </c>
-      <c r="C19" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="D19" s="12" t="s">
-        <v>209</v>
-      </c>
-      <c r="E19" s="20" t="s">
-        <v>195</v>
-      </c>
-      <c r="F19" s="17"/>
+      <c r="A19" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="E19" s="18" t="s">
+        <v>154</v>
+      </c>
+      <c r="F19" s="15"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
@@ -5313,12 +4307,12 @@
       <c r="L19" s="1"/>
     </row>
     <row r="20" spans="1:12" ht="90" customHeight="1">
-      <c r="A20" s="11"/>
-      <c r="B20" s="11"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="17"/>
+      <c r="A20" s="9"/>
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="15"/>
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
@@ -5341,9 +4335,7 @@
       <c r="L21" s="1"/>
     </row>
     <row r="22" spans="1:12" ht="15" customHeight="1">
-      <c r="A22" s="7" t="s">
-        <v>125</v>
-      </c>
+      <c r="A22" s="5"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
@@ -5357,15 +4349,11 @@
       <c r="L22" s="1"/>
     </row>
     <row r="23" spans="1:12" ht="29.1" customHeight="1">
-      <c r="A23" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B23" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="C23" s="8"/>
-      <c r="D23" s="8"/>
-      <c r="E23" s="8"/>
+      <c r="A23" s="1"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
@@ -5375,15 +4363,11 @@
       <c r="L23" s="1"/>
     </row>
     <row r="24" spans="1:12" ht="29.1" customHeight="1">
-      <c r="A24" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="B24" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="C24" s="8"/>
-      <c r="D24" s="8"/>
-      <c r="E24" s="8"/>
+      <c r="A24" s="1"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
@@ -5833,19 +4817,19 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="E7" r:id="rId1" tooltip="Abrir GIF Animado de Evidencia" display="evidencias\sprint1\CP-001_Navegacion_SPA.gif" xr:uid="{E22E884A-8AF5-4E85-80AB-5943303881A5}"/>
-    <hyperlink ref="E8" r:id="rId2" tooltip="Abrir GIF Animado de Evidencia" display="evidencias\sprint1\CP-002_Transicion_Rutas_Hash.gif" xr:uid="{80383DA2-2E61-4C1C-9F7C-D4CE572E220D}"/>
-    <hyperlink ref="E9" r:id="rId3" tooltip="Abrir GIF Animado de Evidencia" display="evidencias\sprint1\CP-003_Exploracion_Inicio.gif" xr:uid="{F988E940-13D6-41A7-AC6B-E93479779C02}"/>
-    <hyperlink ref="E10" r:id="rId4" tooltip="Abrir GIF Animado de Evidencia" display="evidencias\sprint1\CP-004_Animacion_Carrusel.gif" xr:uid="{784CFE2A-9CD6-444E-ADAB-7DDCDCDA3036}"/>
-    <hyperlink ref="E11" r:id="rId5" tooltip="Abrir GIF Animado de Evidencia" display="evidencias\sprint1\CP-005_Navbar_Responsive.gif" xr:uid="{F0C96203-BE6C-4BA5-A8A0-CACAD6F2FC64}"/>
-    <hyperlink ref="E12" r:id="rId6" tooltip="Abrir GIF Animado de Evidencia" display="evidencias\sprint1\CP-006_Contacto_Navegacion.gif" xr:uid="{6861DEF4-8803-4BAD-8681-5DD9AD5FCA5E}"/>
-    <hyperlink ref="E13" r:id="rId7" tooltip="Abrir GIF Animado de Evidencia" display="evidencias\sprint1\CP-007_Toasts_Aparicion.gif" xr:uid="{4A20CDCB-21EB-4102-AC21-D042AB37A8FA}"/>
-    <hyperlink ref="E14" r:id="rId8" tooltip="Abrir GIF Animado de Evidencia" display="evidencias\sprint1\CP-008_Manejo_Rutas_Protegidas.gif" xr:uid="{DAF3516D-2585-4C84-919A-498D5E2C2DB1}"/>
-    <hyperlink ref="E15" r:id="rId9" tooltip="Abrir GIF Animado de Evidencia" display="evidencias\sprint1\CP-009_Carrusel_Teclado.gif" xr:uid="{26665121-9C7D-4BF7-817A-20275B626BA2}"/>
-    <hyperlink ref="E16" r:id="rId10" tooltip="Abrir GIF Animado de Evidencia" display="evidencias\sprint1\CP-0010_Toast_Usabilidad.gif" xr:uid="{C305E022-1700-4F65-A65F-53858FD89B0B}"/>
-    <hyperlink ref="E17" r:id="rId11" tooltip="Abrir GIF Animado de Evidencia" display="evidencias\sprint1\CP-0011_Navegacion_Noticias.gif" xr:uid="{3E5C1E8A-3F5B-4C38-916C-066F04CDD062}"/>
-    <hyperlink ref="E18" r:id="rId12" tooltip="Abrir GIF Animado de Evidencia" display="evidencias\sprint1\CP-0012_Exploracion_Eventos.gif" xr:uid="{4F629DFE-3A5C-40C4-972A-776751C11DF7}"/>
-    <hyperlink ref="E19" r:id="rId13" tooltip="Abrir GIF Animado de Evidencia" display="evidencias\sprint1\CP-0013_Revision_Ediles.gif" xr:uid="{45B3285A-79E5-45EA-AE03-18C43F7493ED}"/>
+    <hyperlink ref="E7" r:id="rId1" tooltip="Abrir GIF Animado de Evidencia" xr:uid="{E22E884A-8AF5-4E85-80AB-5943303881A5}"/>
+    <hyperlink ref="E8" r:id="rId2" tooltip="Abrir GIF Animado de Evidencia" xr:uid="{80383DA2-2E61-4C1C-9F7C-D4CE572E220D}"/>
+    <hyperlink ref="E9" r:id="rId3" tooltip="Abrir GIF Animado de Evidencia" xr:uid="{F988E940-13D6-41A7-AC6B-E93479779C02}"/>
+    <hyperlink ref="E10" r:id="rId4" tooltip="Abrir GIF Animado de Evidencia" xr:uid="{784CFE2A-9CD6-444E-ADAB-7DDCDCDA3036}"/>
+    <hyperlink ref="E11" r:id="rId5" tooltip="Abrir GIF Animado de Evidencia" xr:uid="{F0C96203-BE6C-4BA5-A8A0-CACAD6F2FC64}"/>
+    <hyperlink ref="E12" r:id="rId6" tooltip="Abrir GIF Animado de Evidencia" xr:uid="{6861DEF4-8803-4BAD-8681-5DD9AD5FCA5E}"/>
+    <hyperlink ref="E13" r:id="rId7" tooltip="Abrir GIF Animado de Evidencia" xr:uid="{4A20CDCB-21EB-4102-AC21-D042AB37A8FA}"/>
+    <hyperlink ref="E14" r:id="rId8" tooltip="Abrir GIF Animado de Evidencia" xr:uid="{DAF3516D-2585-4C84-919A-498D5E2C2DB1}"/>
+    <hyperlink ref="E15" r:id="rId9" tooltip="Abrir GIF Animado de Evidencia" xr:uid="{26665121-9C7D-4BF7-817A-20275B626BA2}"/>
+    <hyperlink ref="E16" r:id="rId10" tooltip="Abrir GIF Animado de Evidencia" xr:uid="{C305E022-1700-4F65-A65F-53858FD89B0B}"/>
+    <hyperlink ref="E17" r:id="rId11" tooltip="Abrir GIF Animado de Evidencia" xr:uid="{3E5C1E8A-3F5B-4C38-916C-066F04CDD062}"/>
+    <hyperlink ref="E18" r:id="rId12" tooltip="Abrir GIF Animado de Evidencia" xr:uid="{4F629DFE-3A5C-40C4-972A-776751C11DF7}"/>
+    <hyperlink ref="E19" r:id="rId13" tooltip="Abrir GIF Animado de Evidencia" xr:uid="{45B3285A-79E5-45EA-AE03-18C43F7493ED}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId14"/>

</xml_diff>

<commit_message>
fix(qa): sincronizar enlaces relativos en matriz de pruebas sprint 1
</commit_message>
<xml_diff>
--- a/Plantilla_pruebas_JAL-E01.xlsx
+++ b/Plantilla_pruebas_JAL-E01.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JUAN ECHAVARRIA\Desktop\Voz local\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Miguel\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0463325D-3B44-4907-B303-0B4EB4F40BDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A0E609CD-0394-4028-ACFB-AD895654EA19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3375" yWindow="3375" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Casos" sheetId="2" r:id="rId1"/>
@@ -18,27 +18,11 @@
     <sheet name="Evidencias" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="210">
   <si>
     <t>Casos de prueba</t>
   </si>
@@ -543,6 +527,9 @@
     <t>Ver GIF Animado (CP-0013_Revision_Ediles.gif)</t>
   </si>
   <si>
+    <t>Juan José Echavarria Castaño</t>
+  </si>
+  <si>
     <t>Estructura base de la SPA, carga de hojas de estilo (Bootstrap 5 y custom CSS), componentes estructurales (#app-navbar, #app-root, #app-footer) e inicialización de módulos ES6 sin recarga de página.</t>
   </si>
   <si>
@@ -699,10 +686,10 @@
     <t>Muestra la lista de ediles con sus nombres, cargos, teléfonos y correos de contacto.</t>
   </si>
   <si>
-    <t>Juan José Echavarría Castaño</t>
-  </si>
-  <si>
-    <t>Miguel Ángel Rodríguez Gutiérrez</t>
+    <t>Juan José Echavavaria</t>
+  </si>
+  <si>
+    <t>Miguel Angel Rodriguez</t>
   </si>
 </sst>
 </file>
@@ -1966,7 +1953,7 @@
         <v>17</v>
       </c>
       <c r="H7" s="17" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="I7" s="17" t="s">
         <v>18</v>
@@ -1998,7 +1985,7 @@
         <v>23</v>
       </c>
       <c r="H8" s="17" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I8" s="17" t="s">
         <v>24</v>
@@ -2030,7 +2017,7 @@
         <v>29</v>
       </c>
       <c r="H9" s="17" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="I9" s="17" t="s">
         <v>30</v>
@@ -2062,7 +2049,7 @@
         <v>36</v>
       </c>
       <c r="H10" s="17" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="I10" s="17" t="s">
         <v>37</v>
@@ -2094,7 +2081,7 @@
         <v>90</v>
       </c>
       <c r="H11" s="17" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="I11" s="17" t="s">
         <v>40</v>
@@ -2126,7 +2113,7 @@
         <v>45</v>
       </c>
       <c r="H12" s="17" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="I12" s="17" t="s">
         <v>46</v>
@@ -2158,7 +2145,7 @@
         <v>51</v>
       </c>
       <c r="H13" s="17" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="I13" s="17" t="s">
         <v>52</v>
@@ -2190,7 +2177,7 @@
         <v>58</v>
       </c>
       <c r="H14" s="17" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="I14" s="17" t="s">
         <v>59</v>
@@ -2222,7 +2209,7 @@
         <v>93</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I15" s="6"/>
       <c r="J15" s="1"/>
@@ -2252,7 +2239,7 @@
         <v>99</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="I16" s="6"/>
       <c r="J16" s="1"/>
@@ -2282,7 +2269,7 @@
         <v>103</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="I17" s="6"/>
       <c r="J17" s="1"/>
@@ -2312,7 +2299,7 @@
         <v>107</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="I18" s="6"/>
       <c r="J18" s="1"/>
@@ -2342,7 +2329,7 @@
         <v>111</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="I19" s="6"/>
       <c r="J19" s="1"/>
@@ -3005,13 +2992,13 @@
         <v>113</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F7" s="11" t="s">
         <v>60</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H7" s="12" t="s">
         <v>114</v>
@@ -3019,7 +3006,7 @@
       <c r="I7" s="10"/>
       <c r="J7" s="10"/>
       <c r="K7" s="10" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="42" customHeight="1">
@@ -3036,13 +3023,13 @@
         <v>113</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>207</v>
+        <v>155</v>
       </c>
       <c r="F8" s="11" t="s">
         <v>60</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H8" s="12" t="s">
         <v>115</v>
@@ -3050,7 +3037,7 @@
       <c r="I8" s="10"/>
       <c r="J8" s="10"/>
       <c r="K8" s="10" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="42" customHeight="1">
@@ -3067,13 +3054,13 @@
         <v>113</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>208</v>
+        <v>155</v>
       </c>
       <c r="F9" s="11" t="s">
         <v>60</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H9" s="12" t="s">
         <v>117</v>
@@ -3081,7 +3068,7 @@
       <c r="I9" s="10"/>
       <c r="J9" s="10"/>
       <c r="K9" s="10" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="42" customHeight="1">
@@ -3098,13 +3085,13 @@
         <v>113</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>207</v>
+        <v>155</v>
       </c>
       <c r="F10" s="11" t="s">
         <v>60</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H10" s="12" t="s">
         <v>119</v>
@@ -3112,7 +3099,7 @@
       <c r="I10" s="10"/>
       <c r="J10" s="10"/>
       <c r="K10" s="10" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="42" customHeight="1">
@@ -3129,13 +3116,13 @@
         <v>113</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>208</v>
+        <v>155</v>
       </c>
       <c r="F11" s="11" t="s">
         <v>60</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="H11" s="12" t="s">
         <v>121</v>
@@ -3143,7 +3130,7 @@
       <c r="I11" s="10"/>
       <c r="J11" s="10"/>
       <c r="K11" s="10" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="42" customHeight="1">
@@ -3160,13 +3147,13 @@
         <v>113</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>208</v>
+        <v>155</v>
       </c>
       <c r="F12" s="11" t="s">
         <v>60</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H12" s="12" t="s">
         <v>123</v>
@@ -3174,7 +3161,7 @@
       <c r="I12" s="10"/>
       <c r="J12" s="10"/>
       <c r="K12" s="10" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="42" customHeight="1">
@@ -3191,13 +3178,13 @@
         <v>113</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>207</v>
+        <v>155</v>
       </c>
       <c r="F13" s="11" t="s">
         <v>60</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="H13" s="12" t="s">
         <v>125</v>
@@ -3205,7 +3192,7 @@
       <c r="I13" s="10"/>
       <c r="J13" s="10"/>
       <c r="K13" s="10" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="42" customHeight="1">
@@ -3222,13 +3209,13 @@
         <v>113</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>207</v>
+        <v>155</v>
       </c>
       <c r="F14" s="11" t="s">
         <v>60</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H14" s="12" t="s">
         <v>127</v>
@@ -3236,7 +3223,7 @@
       <c r="I14" s="10"/>
       <c r="J14" s="10"/>
       <c r="K14" s="10" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="42" customHeight="1">
@@ -3253,13 +3240,13 @@
         <v>113</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F15" s="11" t="s">
         <v>60</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="H15" s="12" t="s">
         <v>130</v>
@@ -3267,7 +3254,7 @@
       <c r="I15" s="10"/>
       <c r="J15" s="10"/>
       <c r="K15" s="10" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="42" customHeight="1">
@@ -3284,13 +3271,13 @@
         <v>113</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="F16" s="11" t="s">
         <v>60</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H16" s="12" t="s">
         <v>132</v>
@@ -3298,7 +3285,7 @@
       <c r="I16" s="10"/>
       <c r="J16" s="10"/>
       <c r="K16" s="10" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="42" customHeight="1">
@@ -3315,13 +3302,13 @@
         <v>113</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>208</v>
+        <v>155</v>
       </c>
       <c r="F17" s="11" t="s">
         <v>60</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="H17" s="12" t="s">
         <v>135</v>
@@ -3329,7 +3316,7 @@
       <c r="I17" s="10"/>
       <c r="J17" s="10"/>
       <c r="K17" s="10" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="42" customHeight="1">
@@ -3346,13 +3333,13 @@
         <v>113</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>208</v>
+        <v>155</v>
       </c>
       <c r="F18" s="11" t="s">
         <v>60</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H18" s="12" t="s">
         <v>137</v>
@@ -3360,7 +3347,7 @@
       <c r="I18" s="10"/>
       <c r="J18" s="10"/>
       <c r="K18" s="10" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="42" customHeight="1">
@@ -3377,13 +3364,13 @@
         <v>113</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>207</v>
+        <v>155</v>
       </c>
       <c r="F19" s="11" t="s">
         <v>60</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="H19" s="12" t="s">
         <v>140</v>
@@ -3391,7 +3378,7 @@
       <c r="I19" s="10"/>
       <c r="J19" s="10"/>
       <c r="K19" s="10" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="36" customHeight="1">
@@ -4005,7 +3992,7 @@
         <v>141</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E7" s="18" t="s">
         <v>142</v>
@@ -4029,7 +4016,7 @@
         <v>141</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E8" s="18" t="s">
         <v>143</v>
@@ -4053,7 +4040,7 @@
         <v>141</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E9" s="18" t="s">
         <v>144</v>
@@ -4077,7 +4064,7 @@
         <v>141</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E10" s="18" t="s">
         <v>145</v>
@@ -4101,7 +4088,7 @@
         <v>141</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E11" s="18" t="s">
         <v>146</v>
@@ -4125,7 +4112,7 @@
         <v>141</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E12" s="18" t="s">
         <v>147</v>
@@ -4149,7 +4136,7 @@
         <v>141</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E13" s="18" t="s">
         <v>148</v>
@@ -4173,7 +4160,7 @@
         <v>141</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E14" s="18" t="s">
         <v>149</v>
@@ -4197,7 +4184,7 @@
         <v>141</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E15" s="18" t="s">
         <v>150</v>
@@ -4221,7 +4208,7 @@
         <v>141</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E16" s="18" t="s">
         <v>151</v>
@@ -4245,7 +4232,7 @@
         <v>141</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E17" s="18" t="s">
         <v>152</v>
@@ -4269,7 +4256,7 @@
         <v>141</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E18" s="18" t="s">
         <v>153</v>
@@ -4293,7 +4280,7 @@
         <v>141</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E19" s="18" t="s">
         <v>154</v>

</xml_diff>